<commit_message>
E1 breadth: provenance audit of the pre-audit corpus
All 36 source URLs fetched on the server; every retained text found in its source.
Corrected provenance fields only (310 logged changes in audit/changes_2026-09-13.csv):
- seed locators held Stage A case ids; replaced with real sections/tables/posts
- seed access dates restored from cases.py
- AutoTap 'participant Pnn' was Excel row minus 2 (73/73); replaced with row/column
- two Google Home section names did not exist; replaced with actual headings
- community titles were researcher labels; replaced with real thread titles
- E1-099 normalization gained the stated 2-minute no-motion condition
Strata, screen_status and R/B labels untouched (still pre-audit). Frozen cases unchanged.
Evaluation HANDOFF: drop stale 'B3/B4 unevaluated' line, add breadth status.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
+++ b/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
@@ -1109,12 +1109,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>blueprint.description; input.no_motion_wait.description; mode; actions</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="AF2" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG2" s="3" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>§V-D, extended-action violation example, applet r_i</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="AF3" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG3" s="3" t="inlineStr">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>§V-D, extended-action violation example, applet r_j</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 520305 (2023-01-18)</t>
+          <t>Home Assistant Community thread 520305: How to set notifications when door is left open?</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>opening post (created 2023-01-17 UTC)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="AF5" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG5" s="3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 783900 (2024-10-20)</t>
+          <t>Home Assistant Community thread 783900: How to automate open door notifications?</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>opening post (created 2024-10-18 UTC)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="AF6" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG6" s="3" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>§III template (g) Event-Event Conditional sample response; same statement in User Study 1 data, Result sheet, Excel row 16, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="AF7" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG7" s="3" t="inlineStr">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>§VI-A Task 11, with the authors' rule explanation</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="AF8" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG8" s="3" t="inlineStr">
@@ -1998,12 +1998,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>Results, trigger/action structure paragraph ('one participant specified')</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="AF9" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG9" s="3" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>Table 1, Task I</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="AF10" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG10" s="3" t="inlineStr">
@@ -2252,12 +2252,12 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>Table 5, Q3</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="AF11" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG11" s="3" t="inlineStr">
@@ -2379,12 +2379,12 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>Table 4, P3</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="AF12" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG12" s="3" t="inlineStr">
@@ -2506,12 +2506,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>C20-O</t>
+          <t>Table 1, Event-Event paradigm, second example (full text: https://par.nsf.gov/servlets/purl/10106413)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="AF13" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG13" s="3" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S5</t>
+          <t>Result sheet, Excel row 4, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="AF14" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG14" s="3" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S6</t>
+          <t>Result sheet, Excel row 4, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="AF15" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG15" s="3" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S7</t>
+          <t>Result sheet, Excel row 4, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="AF16" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG16" s="3" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S8</t>
+          <t>Result sheet, Excel row 6, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="AF17" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG17" s="3" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S1</t>
+          <t>Result sheet, Excel row 7, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="AF18" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG18" s="3" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S2</t>
+          <t>Result sheet, Excel row 8, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="AF19" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG19" s="3" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S3</t>
+          <t>Result sheet, Excel row 8, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="AF20" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG20" s="3" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S4</t>
+          <t>Result sheet, Excel row 8, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="AF21" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG21" s="3" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S9</t>
+          <t>Result sheet, Excel row 8, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="AF22" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG22" s="3" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S10</t>
+          <t>Result sheet, Excel row 8, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="AF23" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG23" s="3" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P08, statement S1</t>
+          <t>Result sheet, Excel row 10, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="AF24" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG24" s="3" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P10, statement S6</t>
+          <t>Result sheet, Excel row 12, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="AF25" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG25" s="3" t="inlineStr">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P11, statement S8</t>
+          <t>Result sheet, Excel row 13, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="AF26" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG26" s="3" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P16, statement S6</t>
+          <t>Result sheet, Excel row 18, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="AF27" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG27" s="3" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P19, statement S2</t>
+          <t>Result sheet, Excel row 21, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="AF28" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG28" s="3" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P24, statement S2</t>
+          <t>Result sheet, Excel row 26, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="AF29" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG29" s="3" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P26, statement S4</t>
+          <t>Result sheet, Excel row 28, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="AF30" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG30" s="3" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P29, statement S10</t>
+          <t>Result sheet, Excel row 31, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="AF31" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG31" s="3" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P46, statement S10</t>
+          <t>Result sheet, Excel row 48, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="AF32" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG32" s="3" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P49, statement S3</t>
+          <t>Result sheet, Excel row 51, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="AF33" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG33" s="3" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P52, statement S2</t>
+          <t>Result sheet, Excel row 54, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="AF34" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG34" s="3" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P58, statement S9</t>
+          <t>Result sheet, Excel row 60, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="AF35" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG35" s="3" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P65, statement S3</t>
+          <t>Result sheet, Excel row 67, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="AF36" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG36" s="3" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="AF37" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG37" s="3" t="inlineStr"/>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="AF38" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG38" s="3" t="inlineStr"/>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="AF39" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG39" s="3" t="inlineStr"/>
@@ -6043,7 +6043,7 @@
       </c>
       <c r="AF40" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG40" s="3" t="inlineStr"/>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="AF41" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG41" s="3" t="inlineStr"/>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="AF42" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG42" s="3" t="inlineStr"/>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="AF43" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG43" s="3" t="inlineStr"/>
@@ -6523,7 +6523,7 @@
       </c>
       <c r="AF44" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG44" s="3" t="inlineStr"/>
@@ -6642,7 +6642,7 @@
       </c>
       <c r="AF45" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG45" s="3" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="AF46" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG46" s="3" t="inlineStr"/>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="AF47" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG47" s="3" t="inlineStr"/>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="AF48" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG48" s="3" t="inlineStr"/>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="AF49" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG49" s="3" t="inlineStr"/>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="AF50" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG50" s="3" t="inlineStr"/>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="AF51" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG51" s="3" t="inlineStr"/>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="AF52" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG52" s="3" t="inlineStr"/>
@@ -7602,7 +7602,7 @@
       </c>
       <c r="AF53" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG53" s="3" t="inlineStr"/>
@@ -7725,7 +7725,7 @@
       </c>
       <c r="AF54" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG54" s="3" t="inlineStr"/>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="AF55" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG55" s="3" t="inlineStr"/>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="AF56" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG56" s="3" t="inlineStr"/>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="AF57" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG57" s="3" t="inlineStr"/>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="AF58" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG58" s="3" t="inlineStr"/>
@@ -8320,7 +8320,7 @@
       </c>
       <c r="AF59" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG59" s="3" t="inlineStr"/>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="AF60" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG60" s="3" t="inlineStr"/>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="AF61" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG61" s="3" t="inlineStr"/>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="AF62" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG62" s="3" t="inlineStr"/>
@@ -8802,7 +8802,7 @@
       </c>
       <c r="AF63" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG63" s="3" t="inlineStr"/>
@@ -8921,7 +8921,7 @@
       </c>
       <c r="AF64" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG64" s="3" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="AF65" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG65" s="3" t="inlineStr"/>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="AF66" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG66" s="3" t="inlineStr"/>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="AF67" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG67" s="3" t="inlineStr"/>
@@ -9401,7 +9401,7 @@
       </c>
       <c r="AF68" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG68" s="3" t="inlineStr"/>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="AF69" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG69" s="3" t="inlineStr"/>
@@ -9643,7 +9643,7 @@
       </c>
       <c r="AF70" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG70" s="3" t="inlineStr"/>
@@ -9762,7 +9762,7 @@
       </c>
       <c r="AF71" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG71" s="3" t="inlineStr"/>
@@ -9887,7 +9887,7 @@
       </c>
       <c r="AF72" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG72" s="3" t="inlineStr"/>
@@ -10006,7 +10006,7 @@
       </c>
       <c r="AF73" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG73" s="3" t="inlineStr"/>
@@ -10125,7 +10125,7 @@
       </c>
       <c r="AF74" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG74" s="3" t="inlineStr"/>
@@ -10154,7 +10154,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Google Home example scripted automations — Morning blinds with suppression</t>
+          <t>Google Home example scripted automations — When I walk through my corridor first time (motion sensor) in the morning open all my blinds and suppress the trigger for 20 hours</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>Section: Morning blinds with suppression</t>
+          <t>Section: When I walk through my corridor first time (motion sensor) in the morning open all my blinds and suppress the trigger for 20 hours</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="AF75" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG75" s="3" t="inlineStr"/>
@@ -10273,7 +10273,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Google Home example scripted automations — Weekday movement notification</t>
+          <t>Google Home example scripted automations — Send a notification when movement is detected at home on a weekday</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>Section: Weekday movement notification</t>
+          <t>Section: Send a notification when movement is detected at home on a weekday</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -10363,7 +10363,7 @@
       </c>
       <c r="AF76" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG76" s="3" t="inlineStr"/>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="AF77" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG77" s="3" t="inlineStr"/>
@@ -10601,7 +10601,7 @@
       </c>
       <c r="AF78" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG78" s="3" t="inlineStr"/>
@@ -10640,7 +10640,7 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-03-14 UTC)</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -10720,7 +10720,7 @@
       </c>
       <c r="AF79" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG79" s="3" t="inlineStr"/>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 864628: Trigger automation every minute unless sensor updates</t>
+          <t>Home Assistant Community thread 864628: Trigger automation every minute, unless it has been triggered by something else</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-03-16 UTC)</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="AF80" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG80" s="3" t="inlineStr"/>
@@ -10868,7 +10868,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 408113: Arm alarm when everyone is away</t>
+          <t>Home Assistant Community thread 408113: Automation - Arm Alarm when everyone is away?</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2022-04-03 UTC)</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -10958,7 +10958,7 @@
       </c>
       <c r="AF81" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG81" s="3" t="inlineStr"/>
@@ -10987,7 +10987,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 721406: Repeat movement reminder</t>
+          <t>Home Assistant Community thread 721406: How to reliably design making an announcement every 5 mins until a binary sensor is OFF</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -10997,7 +10997,7 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-04-24 UTC)</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="AF82" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG82" s="3" t="inlineStr"/>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 600389: Notify when a long-open door closes</t>
+          <t>Home Assistant Community thread 600389: Help with Door Close Automation</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-08-07 UTC)</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -11196,7 +11196,7 @@
       </c>
       <c r="AF83" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG83" s="3" t="inlineStr"/>
@@ -11225,7 +11225,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 958200: Temporary automation override</t>
+          <t>Home Assistant Community thread 958200: Delayed entity, AKA "turn this on for X minutes"</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-12-03 UTC)</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="AF84" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG84" s="3" t="inlineStr"/>
@@ -11352,7 +11352,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 566330: Different weekday/weekend light schedules</t>
+          <t>Home Assistant Community thread 566330: Automation to turn ON/OFF devices at different times/days</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-05-01 UTC)</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="AF85" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG85" s="3" t="inlineStr"/>
@@ -11471,7 +11471,7 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 485629: Temperature hysteresis</t>
+          <t>Home Assistant Community thread 485629: How to trigger an automation based on temperature hysteresis</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -11481,7 +11481,7 @@
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2022-11-07 UTC)</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -11561,7 +11561,7 @@
       </c>
       <c r="AF86" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG86" s="3" t="inlineStr"/>
@@ -11590,7 +11590,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 878961: Cancelable sequential sprinklers</t>
+          <t>Home Assistant Community thread 878961: Stop an automation mid-run via an input boolean?</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-04-17 UTC)</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="AF87" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG87" s="3" t="inlineStr"/>
@@ -11715,7 +11715,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 367362: Restartable ten-minute light</t>
+          <t>Home Assistant Community thread 367362: Understanding automations with time delays and how to control them</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -11725,7 +11725,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2021-12-15 UTC)</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="AF88" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG88" s="3" t="inlineStr"/>
@@ -11838,7 +11838,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 712624: Early lights for dark weather</t>
+          <t>Home Assistant Community thread 712624: How to enable an automation between times</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-04-03 UTC)</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="AF89" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG89" s="3" t="inlineStr"/>
@@ -11957,7 +11957,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 302465: Exterior light around sunset/sunrise</t>
+          <t>Home Assistant Community thread 302465: Evolution of an automation. Turn a light on/off at sunset/sunrise</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2021-04-24 UTC)</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="AF90" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG90" s="3" t="inlineStr"/>
@@ -12076,7 +12076,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 670621: Turn on for a set time</t>
+          <t>Home Assistant Community thread 670621: Turn something on for a set time</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -12086,7 +12086,7 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-01-10 UTC)</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -12170,7 +12170,7 @@
       </c>
       <c r="AF91" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG91" s="3" t="inlineStr"/>
@@ -12199,7 +12199,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 987759: Periodic multi-valve check</t>
+          <t>Home Assistant Community thread 987759: Automation to run every 5 minutes</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -12209,7 +12209,7 @@
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-02-17 UTC)</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -12297,7 +12297,7 @@
       </c>
       <c r="AF92" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG92" s="3" t="inlineStr"/>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 955561: Independent parallel shutdown flows</t>
+          <t>Home Assistant Community thread 955561: Running groups of actions in Parallel</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-11-26 UTC)</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="AF93" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG93" s="3" t="inlineStr"/>
@@ -12455,7 +12455,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 555703: Parallel doorbell displays</t>
+          <t>Home Assistant Community thread 555703: [solved] Automation w/ 3 actions (notification scripts): how to make them run in parallel?</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -12465,7 +12465,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-04-03 UTC)</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="AF94" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG94" s="3" t="inlineStr"/>
@@ -12578,7 +12578,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 585191: Parallel light sequences</t>
+          <t>Home Assistant Community thread 585191: Trying to create action in parallel with delays for certain actions that need to occur sequentially</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -12588,7 +12588,7 @@
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-06-24 UTC)</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -12672,7 +12672,7 @@
       </c>
       <c r="AF95" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG95" s="3" t="inlineStr"/>
@@ -12701,7 +12701,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 654561: Pool reading averages</t>
+          <t>Home Assistant Community thread 654561: Getting an average reading of a sensor during certain hours</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-12 UTC)</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="AF96" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG96" s="3" t="inlineStr"/>
@@ -12834,7 +12834,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 653754: Low battery report</t>
+          <t>Home Assistant Community thread 653754: 🪫 Low Battery Notifications &amp; Actions</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-11 UTC)</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="AF97" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG97" s="3" t="inlineStr"/>
@@ -12953,7 +12953,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 892319: Presence-aware doorbell actions</t>
+          <t>Home Assistant Community thread 892319: 🔔 Smart Doorbell Button (Zigbee) with Sound, Lights, Notifications &amp; Presence Awareness</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-05-19 UTC)</t>
         </is>
       </c>
       <c r="I98" s="3" t="inlineStr">
@@ -13047,7 +13047,7 @@
       </c>
       <c r="AF98" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG98" s="3" t="inlineStr"/>
@@ -13076,7 +13076,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 1024799: Washing-machine finished notification</t>
+          <t>Home Assistant Community thread 1024799: Simple Washing Machine Finished Notification – power sensor + helper, beginner friendly</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -13086,7 +13086,7 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-09-12 UTC)</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="AF99" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG99" s="3" t="inlineStr"/>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 729908: Manual light with minimum-on and motion extension</t>
+          <t>Home Assistant Community thread 729908: Need help with light automation</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-05-16 UTC)</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes.</t>
+          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes; the light is turned off only when no motion has been detected for 2 minutes.</t>
         </is>
       </c>
       <c r="K100" s="3" t="inlineStr"/>
@@ -13291,7 +13291,7 @@
       </c>
       <c r="AF100" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG100" s="3" t="inlineStr"/>
@@ -13320,7 +13320,7 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 641504: Last resident leaves and door unlocked</t>
+          <t>Home Assistant Community thread 641504: Automation that triggers when all residents are not home</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-11-16 UTC)</t>
         </is>
       </c>
       <c r="I101" s="3" t="inlineStr">
@@ -13410,7 +13410,7 @@
       </c>
       <c r="AF101" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG101" s="3" t="inlineStr"/>
@@ -13776,12 +13776,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>blueprint.description; input.no_motion_wait.description; mode; actions</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="AF2" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG2" s="3" t="inlineStr">
@@ -13903,12 +13903,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>§V-D, extended-action violation example, applet r_i</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="AF3" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG3" s="3" t="inlineStr">
@@ -14030,12 +14030,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>§V-D, extended-action violation example, applet r_j</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -14110,7 +14110,7 @@
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 520305 (2023-01-18)</t>
+          <t>Home Assistant Community thread 520305: How to set notifications when door is left open?</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -14157,12 +14157,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>opening post (created 2023-01-17 UTC)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="AF5" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG5" s="3" t="inlineStr">
@@ -14274,7 +14274,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 783900 (2024-10-20)</t>
+          <t>Home Assistant Community thread 783900: How to automate open door notifications?</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -14284,12 +14284,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>opening post (created 2024-10-18 UTC)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="AF6" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG6" s="3" t="inlineStr">
@@ -14411,12 +14411,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>§III template (g) Event-Event Conditional sample response; same statement in User Study 1 data, Result sheet, Excel row 16, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -14491,7 +14491,7 @@
       </c>
       <c r="AF7" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG7" s="3" t="inlineStr">
@@ -14538,12 +14538,12 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>§VI-A Task 11, with the authors' rule explanation</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="AF8" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG8" s="3" t="inlineStr">
@@ -14665,12 +14665,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>Results, trigger/action structure paragraph ('one participant specified')</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -14745,7 +14745,7 @@
       </c>
       <c r="AF9" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG9" s="3" t="inlineStr">
@@ -14792,12 +14792,12 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>Table 1, Task I</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -14872,7 +14872,7 @@
       </c>
       <c r="AF10" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG10" s="3" t="inlineStr">
@@ -14919,12 +14919,12 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>Table 5, Q3</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="AF11" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG11" s="3" t="inlineStr">
@@ -15046,12 +15046,12 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>Table 4, P3</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -15126,7 +15126,7 @@
       </c>
       <c r="AF12" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG12" s="3" t="inlineStr">
@@ -15173,12 +15173,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>C20-O</t>
+          <t>Table 1, Event-Event paradigm, second example (full text: https://par.nsf.gov/servlets/purl/10106413)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="AF13" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG13" s="3" t="inlineStr">
@@ -15286,7 +15286,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 955561: Independent parallel shutdown flows</t>
+          <t>Home Assistant Community thread 955561: Running groups of actions in Parallel</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -15296,7 +15296,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-11-26 UTC)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -15386,7 +15386,7 @@
       </c>
       <c r="AF14" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG14" s="3" t="inlineStr"/>
@@ -15415,7 +15415,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 654561: Pool reading averages</t>
+          <t>Home Assistant Community thread 654561: Getting an average reading of a sensor during certain hours</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -15425,7 +15425,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-12 UTC)</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -15519,7 +15519,7 @@
       </c>
       <c r="AF15" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG15" s="3" t="inlineStr"/>
@@ -15548,7 +15548,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 878961: Cancelable sequential sprinklers</t>
+          <t>Home Assistant Community thread 878961: Stop an automation mid-run via an input boolean?</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-04-17 UTC)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -15644,7 +15644,7 @@
       </c>
       <c r="AF16" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG16" s="3" t="inlineStr"/>
@@ -15673,7 +15673,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 729908: Manual light with minimum-on and motion extension</t>
+          <t>Home Assistant Community thread 729908: Need help with light automation</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -15683,7 +15683,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-05-16 UTC)</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes.</t>
+          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes; the light is turned off only when no motion has been detected for 2 minutes.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr"/>
@@ -15769,7 +15769,7 @@
       </c>
       <c r="AF17" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG17" s="3" t="inlineStr"/>
@@ -15808,7 +15808,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P24, statement S2</t>
+          <t>Result sheet, Excel row 26, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -15898,7 +15898,7 @@
       </c>
       <c r="AF18" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG18" s="3" t="inlineStr">
@@ -15941,7 +15941,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P58, statement S9</t>
+          <t>Result sheet, Excel row 60, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="AF19" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG19" s="3" t="inlineStr">
@@ -16160,7 +16160,7 @@
       </c>
       <c r="AF20" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG20" s="3" t="inlineStr"/>
@@ -16285,7 +16285,7 @@
       </c>
       <c r="AF21" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG21" s="3" t="inlineStr"/>
@@ -16567,7 +16567,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S7</t>
+          <t>Result sheet, Excel row 4, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="AF2" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG2" s="3" t="inlineStr">
@@ -16702,7 +16702,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S1</t>
+          <t>Result sheet, Excel row 7, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -16794,7 +16794,7 @@
       </c>
       <c r="AF3" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG3" s="3" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S2</t>
+          <t>Result sheet, Excel row 8, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
@@ -16972,7 +16972,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P46, statement S10</t>
+          <t>Result sheet, Excel row 48, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -17064,7 +17064,7 @@
       </c>
       <c r="AF5" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG5" s="3" t="inlineStr">
@@ -17191,7 +17191,7 @@
       </c>
       <c r="AF6" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG6" s="3" t="inlineStr"/>
@@ -17314,7 +17314,7 @@
       </c>
       <c r="AF7" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13</t>
         </is>
       </c>
       <c r="AG7" s="3" t="inlineStr"/>
@@ -17343,7 +17343,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 958200: Temporary automation override</t>
+          <t>Home Assistant Community thread 958200: Delayed entity, AKA "turn this on for X minutes"</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -17353,7 +17353,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-12-03 UTC)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -17441,7 +17441,7 @@
       </c>
       <c r="AF8" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG8" s="3" t="inlineStr"/>
@@ -17470,7 +17470,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 987759: Periodic multi-valve check</t>
+          <t>Home Assistant Community thread 987759: Automation to run every 5 minutes</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -17480,7 +17480,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-02-17 UTC)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -17568,7 +17568,7 @@
       </c>
       <c r="AF9" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG9" s="3" t="inlineStr"/>
@@ -17597,7 +17597,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Home Assistant Community thread 654561: Pool reading averages</t>
+          <t>Home Assistant Community thread 654561: Getting an average reading of a sensor during certain hours</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-12 UTC)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -17701,7 +17701,7 @@
       </c>
       <c r="AF10" s="3" t="inlineStr">
         <is>
-          <t>SOURCE_AND_LOCATOR_CHECKED</t>
+          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
       <c r="AG10" s="3" t="inlineStr"/>
@@ -17810,7 +17810,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>blueprint.description; input.no_motion_wait.description; mode; actions</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -17847,7 +17847,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>§V-D, extended-action violation example, applet r_i</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -17884,7 +17884,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>§V-D, extended-action violation example, applet r_j</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -17921,7 +17921,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>opening post (created 2023-01-17 UTC)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -17958,7 +17958,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>opening post (created 2024-10-18 UTC)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -17995,7 +17995,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>§III template (g) Event-Event Conditional sample response; same statement in User Study 1 data, Result sheet, Excel row 16, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -18032,7 +18032,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>§VI-A Task 11, with the authors' rule explanation</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -18069,7 +18069,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>Results, trigger/action structure paragraph ('one participant specified')</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>Table 1, Task I</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -18143,7 +18143,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>Table 5, Q3</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>Table 4, P3</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -18217,7 +18217,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>C20-O</t>
+          <t>Table 1, Event-Event paradigm, second example (full text: https://par.nsf.gov/servlets/purl/10106413)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -18254,7 +18254,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S5</t>
+          <t>Result sheet, Excel row 4, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -18291,7 +18291,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S6</t>
+          <t>Result sheet, Excel row 4, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -18328,7 +18328,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S7</t>
+          <t>Result sheet, Excel row 4, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -18365,7 +18365,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S8</t>
+          <t>Result sheet, Excel row 6, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S1</t>
+          <t>Result sheet, Excel row 7, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -18439,7 +18439,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S2</t>
+          <t>Result sheet, Excel row 8, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -18476,7 +18476,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S3</t>
+          <t>Result sheet, Excel row 8, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -18513,7 +18513,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S4</t>
+          <t>Result sheet, Excel row 8, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -18550,7 +18550,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S9</t>
+          <t>Result sheet, Excel row 8, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -18587,7 +18587,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S10</t>
+          <t>Result sheet, Excel row 8, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -18624,7 +18624,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P08, statement S1</t>
+          <t>Result sheet, Excel row 10, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -18661,7 +18661,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P10, statement S6</t>
+          <t>Result sheet, Excel row 12, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -18698,7 +18698,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P11, statement S8</t>
+          <t>Result sheet, Excel row 13, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P16, statement S6</t>
+          <t>Result sheet, Excel row 18, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -18772,7 +18772,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P19, statement S2</t>
+          <t>Result sheet, Excel row 21, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -18809,7 +18809,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P24, statement S2</t>
+          <t>Result sheet, Excel row 26, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P26, statement S4</t>
+          <t>Result sheet, Excel row 28, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -18883,7 +18883,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P29, statement S10</t>
+          <t>Result sheet, Excel row 31, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -18920,7 +18920,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P46, statement S10</t>
+          <t>Result sheet, Excel row 48, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -18957,7 +18957,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P49, statement S3</t>
+          <t>Result sheet, Excel row 51, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -18994,7 +18994,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P52, statement S2</t>
+          <t>Result sheet, Excel row 54, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -19031,7 +19031,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P58, statement S9</t>
+          <t>Result sheet, Excel row 60, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P65, statement S3</t>
+          <t>Result sheet, Excel row 67, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -20511,7 +20511,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Section: Morning blinds with suppression</t>
+          <t>Section: When I walk through my corridor first time (motion sensor) in the morning open all my blinds and suppress the trigger for 20 hours</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -20548,7 +20548,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Section: Weekday movement notification</t>
+          <t>Section: Send a notification when movement is detected at home on a weekday</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -20659,7 +20659,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-03-14 UTC)</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -20696,7 +20696,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-03-16 UTC)</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -20733,7 +20733,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2022-04-03 UTC)</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -20770,7 +20770,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-04-24 UTC)</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -20807,7 +20807,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-08-07 UTC)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -20844,7 +20844,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-12-03 UTC)</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -20881,7 +20881,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-05-01 UTC)</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -20918,7 +20918,7 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2022-11-07 UTC)</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
@@ -20955,7 +20955,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-04-17 UTC)</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -20992,7 +20992,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2021-12-15 UTC)</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -21029,7 +21029,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-04-03 UTC)</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -21066,7 +21066,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2021-04-24 UTC)</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -21103,7 +21103,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-01-10 UTC)</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
@@ -21140,7 +21140,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-02-17 UTC)</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
@@ -21177,7 +21177,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-11-26 UTC)</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -21214,7 +21214,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-04-03 UTC)</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
@@ -21251,7 +21251,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-06-24 UTC)</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-12 UTC)</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
@@ -21325,7 +21325,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-12-11 UTC)</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
@@ -21362,7 +21362,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2025-05-19 UTC)</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2026-09-12 UTC)</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
@@ -21436,12 +21436,12 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2024-05-16 UTC)</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes.</t>
+          <t>A manually switched-on light stays on at least 5 minutes; each motion event extends the on time by 2 minutes; the light is turned off only when no motion has been detected for 2 minutes.</t>
         </is>
       </c>
     </row>
@@ -21473,7 +21473,7 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>opening post / stated desired behavior</t>
+          <t>opening post (created 2023-11-16 UTC)</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
@@ -21506,7 +21506,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S1</t>
+          <t>Result sheet, Excel row 3, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
@@ -21539,7 +21539,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S2</t>
+          <t>Result sheet, Excel row 3, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
@@ -21572,7 +21572,7 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S3</t>
+          <t>Result sheet, Excel row 3, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
@@ -21605,7 +21605,7 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S4</t>
+          <t>Result sheet, Excel row 3, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
@@ -21638,7 +21638,7 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S5</t>
+          <t>Result sheet, Excel row 3, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
@@ -21671,7 +21671,7 @@
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S6</t>
+          <t>Result sheet, Excel row 3, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
@@ -21704,7 +21704,7 @@
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S7</t>
+          <t>Result sheet, Excel row 3, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr">
@@ -21737,7 +21737,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S8</t>
+          <t>Result sheet, Excel row 3, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -21770,7 +21770,7 @@
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S9</t>
+          <t>Result sheet, Excel row 3, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr">
@@ -21803,7 +21803,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P01, statement S10</t>
+          <t>Result sheet, Excel row 3, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -21836,7 +21836,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S1</t>
+          <t>Result sheet, Excel row 4, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S2</t>
+          <t>Result sheet, Excel row 4, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -21902,7 +21902,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S3</t>
+          <t>Result sheet, Excel row 4, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
@@ -21935,7 +21935,7 @@
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S4</t>
+          <t>Result sheet, Excel row 4, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr">
@@ -21968,7 +21968,7 @@
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S8</t>
+          <t>Result sheet, Excel row 4, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -22001,7 +22001,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S9</t>
+          <t>Result sheet, Excel row 4, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -22034,7 +22034,7 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P02, statement S10</t>
+          <t>Result sheet, Excel row 4, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G118" s="3" t="inlineStr">
@@ -22067,7 +22067,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S1</t>
+          <t>Result sheet, Excel row 6, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -22100,7 +22100,7 @@
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S2</t>
+          <t>Result sheet, Excel row 6, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G120" s="3" t="inlineStr">
@@ -22133,7 +22133,7 @@
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S3</t>
+          <t>Result sheet, Excel row 6, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G121" s="3" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S4</t>
+          <t>Result sheet, Excel row 6, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G122" s="3" t="inlineStr">
@@ -22199,7 +22199,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S5</t>
+          <t>Result sheet, Excel row 6, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr">
@@ -22232,7 +22232,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S6</t>
+          <t>Result sheet, Excel row 6, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S7</t>
+          <t>Result sheet, Excel row 6, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G125" s="3" t="inlineStr">
@@ -22298,7 +22298,7 @@
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S9</t>
+          <t>Result sheet, Excel row 6, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G126" s="3" t="inlineStr">
@@ -22331,7 +22331,7 @@
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P04, statement S10</t>
+          <t>Result sheet, Excel row 6, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G127" s="3" t="inlineStr">
@@ -22364,7 +22364,7 @@
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S2</t>
+          <t>Result sheet, Excel row 7, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S3</t>
+          <t>Result sheet, Excel row 7, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
@@ -22430,7 +22430,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S4</t>
+          <t>Result sheet, Excel row 7, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
@@ -22463,7 +22463,7 @@
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S5</t>
+          <t>Result sheet, Excel row 7, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
@@ -22496,7 +22496,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S6</t>
+          <t>Result sheet, Excel row 7, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -22529,7 +22529,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S7</t>
+          <t>Result sheet, Excel row 7, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -22562,7 +22562,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S8</t>
+          <t>Result sheet, Excel row 7, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G134" s="3" t="inlineStr">
@@ -22595,7 +22595,7 @@
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S9</t>
+          <t>Result sheet, Excel row 7, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr">
@@ -22628,7 +22628,7 @@
       </c>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P05, statement S10</t>
+          <t>Result sheet, Excel row 7, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G136" s="3" t="inlineStr">
@@ -22661,7 +22661,7 @@
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S1</t>
+          <t>Result sheet, Excel row 8, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G137" s="3" t="inlineStr">
@@ -22694,7 +22694,7 @@
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S5</t>
+          <t>Result sheet, Excel row 8, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G138" s="3" t="inlineStr">
@@ -22727,7 +22727,7 @@
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S6</t>
+          <t>Result sheet, Excel row 8, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G139" s="3" t="inlineStr">
@@ -22760,7 +22760,7 @@
       </c>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S7</t>
+          <t>Result sheet, Excel row 8, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G140" s="3" t="inlineStr">
@@ -22793,7 +22793,7 @@
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P06, statement S8</t>
+          <t>Result sheet, Excel row 8, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
@@ -22826,7 +22826,7 @@
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S1</t>
+          <t>Result sheet, Excel row 9, column AM (header 1_Q25, statement 1)</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr">
@@ -22859,7 +22859,7 @@
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S2</t>
+          <t>Result sheet, Excel row 9, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
@@ -22892,7 +22892,7 @@
       </c>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S3</t>
+          <t>Result sheet, Excel row 9, column AW (header 3_Q25, statement 3)</t>
         </is>
       </c>
       <c r="G144" s="3" t="inlineStr">
@@ -22925,7 +22925,7 @@
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S4</t>
+          <t>Result sheet, Excel row 9, column BB (header 4_Q25, statement 4)</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr">
@@ -22958,7 +22958,7 @@
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S5</t>
+          <t>Result sheet, Excel row 9, column BG (header 5_Q25, statement 5)</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
@@ -22991,7 +22991,7 @@
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S6</t>
+          <t>Result sheet, Excel row 9, column BL (header 6_Q25, statement 6)</t>
         </is>
       </c>
       <c r="G147" s="3" t="inlineStr">
@@ -23024,7 +23024,7 @@
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S7</t>
+          <t>Result sheet, Excel row 9, column BQ (header 7_Q25, statement 7)</t>
         </is>
       </c>
       <c r="G148" s="3" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S8</t>
+          <t>Result sheet, Excel row 9, column BV (header 8_Q25, statement 8)</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr">
@@ -23090,7 +23090,7 @@
       </c>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S9</t>
+          <t>Result sheet, Excel row 9, column CA (header 9_Q25, statement 9)</t>
         </is>
       </c>
       <c r="G150" s="3" t="inlineStr">
@@ -23123,7 +23123,7 @@
       </c>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, participant P07, statement S10</t>
+          <t>Result sheet, Excel row 9, column CF (header 10_Q25, statement 10)</t>
         </is>
       </c>
       <c r="G151" s="3" t="inlineStr">

</xml_diff>

<commit_message>
E1 breadth: apply corpus decisions; freeze depth transcription before encoding
- C15 (E1-008) reclassified elicited -> research; corpus reported as source-diverse
  (official 25 / research 26 / elicited 24 / community 25), no fixed per-stratum quota
- single-author manual screening and R/B coding; no second coder or kappa claimed
- removed root zip and outdated handoff/protocol copies (logged in audit/CLEANUP_2026-09-13.md)
- depth/depth_cases.py: IR-free executable transcription of the eight frozen cases with
  uniform rules T1-T7 (time origin, pulses, unordered same-time comparison, fault injection)
- depth/fixture.py: E1-local typed leaf stubs; global catalog untouched

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
+++ b/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
@@ -812,7 +812,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>• 25 items per source stratum: official, research, elicited, community.</t>
+          <t>• Source-diverse corpus: official 25, research 26, elicited 24, community 25 (C15 reclassified after audit; no rebalancing).</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>• rb_preliminary is triage only; two independent coder columns and adjudicated labels remain blank.</t>
+          <t>• rb_preliminary is machine-assisted triage only. The author screens and codes manually; no second coder or kappa is used. Final labels remain blank until the author enters them.</t>
         </is>
       </c>
     </row>
@@ -1978,12 +1978,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>elicited</t>
+          <t>research</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>user-study elicited</t>
+          <t>paper-reported participant quote</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -14645,12 +14645,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>elicited</t>
+          <t>research</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>user-study elicited</t>
+          <t>paper-reported participant quote</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
E1 breadth: apply author manual screening of the 100-item corpus
- screen_status: 92 IN_SCOPE / 6 AMBIGUOUS / 2 OUT_OF_SCOPE / 0 UNMATCHED
  (E1-031 and E1-095 to IN_SCOPE, E1-027 to AMBIGUOUS); interpretations in notes
- duplicate_family cleared (no retained duplicate); similar topics kept in topic_family
- class-column corrections as stated by the author; rb_adjudicated for 8 rows
  whose R/B set follows from the statement; the rest stays open
- record audit/AUTHOR_SCREENING_2026-09-13.md, change log (55), workbook rebuilt

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPrygyUUKfHFM8zKEvmbin
</commit_message>
<xml_diff>
--- a/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
+++ b/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Corpus_100'!$A$1:$AG$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Depth_20'!$A$1:$AG$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ambiguity_Queue'!$A$1:$AG$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Corpus_100'!$A$1:$AH$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Depth_20'!$A$1:$AH$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Ambiguity_Queue'!$A$1:$AH$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Screening_150'!$A$1:$G$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -172,9 +172,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Corpus100" displayName="Corpus100" ref="A1:AG101" headerRowCount="1">
-  <autoFilter ref="A1:AG101"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Corpus100" displayName="Corpus100" ref="A1:AH101" headerRowCount="1">
+  <autoFilter ref="A1:AH101"/>
+  <tableColumns count="34">
     <tableColumn id="1" name="corpus_id"/>
     <tableColumn id="2" name="cohort"/>
     <tableColumn id="3" name="prior_case_id"/>
@@ -208,15 +208,16 @@
     <tableColumn id="31" name="text_form"/>
     <tableColumn id="32" name="source_verification"/>
     <tableColumn id="33" name="notes"/>
+    <tableColumn id="34" name="topic_family"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Depth20" displayName="Depth20" ref="A1:AG21" headerRowCount="1">
-  <autoFilter ref="A1:AG21"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Depth20" displayName="Depth20" ref="A1:AH21" headerRowCount="1">
+  <autoFilter ref="A1:AH21"/>
+  <tableColumns count="34">
     <tableColumn id="1" name="corpus_id"/>
     <tableColumn id="2" name="cohort"/>
     <tableColumn id="3" name="prior_case_id"/>
@@ -250,15 +251,16 @@
     <tableColumn id="31" name="text_form"/>
     <tableColumn id="32" name="source_verification"/>
     <tableColumn id="33" name="notes"/>
+    <tableColumn id="34" name="topic_family"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AmbiguityQueue" displayName="AmbiguityQueue" ref="A1:AG10" headerRowCount="1">
-  <autoFilter ref="A1:AG10"/>
-  <tableColumns count="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AmbiguityQueue" displayName="AmbiguityQueue" ref="A1:AH9" headerRowCount="1">
+  <autoFilter ref="A1:AH9"/>
+  <tableColumns count="34">
     <tableColumn id="1" name="corpus_id"/>
     <tableColumn id="2" name="cohort"/>
     <tableColumn id="3" name="prior_case_id"/>
@@ -292,6 +294,7 @@
     <tableColumn id="31" name="text_form"/>
     <tableColumn id="32" name="source_verification"/>
     <tableColumn id="33" name="notes"/>
+    <tableColumn id="34" name="topic_family"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
 </table>
@@ -625,7 +628,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e1-corpus-v0.1-preaudit</t>
+          <t>e1-corpus-v0.2-author-screened</t>
         </is>
       </c>
     </row>
@@ -833,7 +836,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>• rb_preliminary is machine-assisted triage only. The author screens and codes manually; no second coder or kappa is used. Final labels remain blank until the author enters them.</t>
+          <t>• Screening status is the author's manual screening (2026-09-13); no retained duplicate. No second coder or kappa is used. rb_preliminary is triage only; rb_adjudicated holds the author's R/B labels and is incomplete.</t>
         </is>
       </c>
     </row>
@@ -866,7 +869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG101"/>
+  <dimension ref="A1:AH101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -902,6 +905,7 @@
     <col width="24" customWidth="1" min="31" max="31"/>
     <col width="24" customWidth="1" min="32" max="32"/>
     <col width="42" customWidth="1" min="33" max="33"/>
+    <col width="15" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1068,6 +1072,11 @@
       <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>topic_family</t>
         </is>
       </c>
     </row>
@@ -1197,6 +1206,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1324,6 +1334,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1451,6 +1462,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1578,6 +1590,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1705,6 +1718,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1832,6 +1846,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1959,6 +1974,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -2086,6 +2102,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -2213,6 +2230,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -2340,6 +2358,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -2467,6 +2486,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2594,6 +2614,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -2721,6 +2742,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2848,6 +2870,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2983,6 +3006,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3110,6 +3134,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -3245,6 +3270,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH18" s="3" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -3380,6 +3406,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH19" s="3" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -3507,6 +3534,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -3631,9 +3659,10 @@
       </c>
       <c r="AG21" s="3" t="inlineStr">
         <is>
-          <t>Original spelling preserved.</t>
-        </is>
-      </c>
+          <t>Original spelling preserved. Author interpretation: if one of the two appliances is already running, a later start request for the other is not started. No notification action is added.</t>
+        </is>
+      </c>
+      <c r="AH21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -3761,6 +3790,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH22" s="3" t="inlineStr"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -3888,6 +3918,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH23" s="3" t="inlineStr"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -4015,6 +4046,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -4142,6 +4174,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -4269,6 +4302,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -4396,6 +4430,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -4451,10 +4486,14 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>IN_SCOPE</t>
-        </is>
-      </c>
-      <c r="M28" s="3" t="inlineStr"/>
+          <t>AMBIGUOUS</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>The clock meaning of 'between 7 and 12 pm' is unclear; the original text is kept without normalization.</t>
+        </is>
+      </c>
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
@@ -4506,7 +4545,11 @@
       </c>
       <c r="AA28" s="3" t="inlineStr"/>
       <c r="AB28" s="3" t="inlineStr"/>
-      <c r="AC28" s="3" t="inlineStr"/>
+      <c r="AC28" s="3" t="inlineStr">
+        <is>
+          <t>Which time range 'between 7 and 12 pm' denotes.</t>
+        </is>
+      </c>
       <c r="AD28" s="3" t="inlineStr"/>
       <c r="AE28" s="3" t="inlineStr">
         <is>
@@ -4523,6 +4566,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH28" s="3" t="inlineStr"/>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -4656,6 +4700,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH29" s="3" t="inlineStr"/>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -4783,6 +4828,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH30" s="3" t="inlineStr"/>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -4910,6 +4956,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
@@ -4965,14 +5012,10 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>UNMATCHED</t>
-        </is>
-      </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Clear daily-count requirement, but the current service catalog does not expose the required history/count value.</t>
-        </is>
-      </c>
+          <t>IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr"/>
       <c r="O32" s="3" t="inlineStr">
         <is>
@@ -5042,9 +5085,10 @@
       </c>
       <c r="AG32" s="3" t="inlineStr">
         <is>
-          <t>Original spelling preserved.</t>
-        </is>
-      </c>
+          <t>Original spelling preserved. Author interpretation: a backend history/count service provides the day's toothbrush use count and the automation reads it as a guard. This is not a claim that the IR performs internal accumulation.</t>
+        </is>
+      </c>
+      <c r="AH32" s="3" t="inlineStr"/>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
@@ -5172,6 +5216,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -5299,6 +5344,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH34" s="3" t="inlineStr"/>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
@@ -5432,6 +5478,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH35" s="3" t="inlineStr"/>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
@@ -5559,6 +5606,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -5682,6 +5730,7 @@
         </is>
       </c>
       <c r="AG37" s="3" t="inlineStr"/>
+      <c r="AH37" s="3" t="inlineStr"/>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
@@ -5805,6 +5854,7 @@
         </is>
       </c>
       <c r="AG38" s="3" t="inlineStr"/>
+      <c r="AH38" s="3" t="inlineStr"/>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -5924,6 +5974,7 @@
         </is>
       </c>
       <c r="AG39" s="3" t="inlineStr"/>
+      <c r="AH39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -5979,11 +6030,7 @@
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="3" t="inlineStr">
-        <is>
-          <t>lights/sun</t>
-        </is>
-      </c>
+      <c r="N40" s="3" t="inlineStr"/>
       <c r="O40" s="3" t="inlineStr">
         <is>
           <t>event/state</t>
@@ -6047,6 +6094,11 @@
         </is>
       </c>
       <c r="AG40" s="3" t="inlineStr"/>
+      <c r="AH40" s="3" t="inlineStr">
+        <is>
+          <t>lights/sun</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -6102,11 +6154,7 @@
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr">
-        <is>
-          <t>lights/sun</t>
-        </is>
-      </c>
+      <c r="N41" s="3" t="inlineStr"/>
       <c r="O41" s="3" t="inlineStr">
         <is>
           <t>event/state; clock/calendar</t>
@@ -6170,6 +6218,11 @@
         </is>
       </c>
       <c r="AG41" s="3" t="inlineStr"/>
+      <c r="AH41" s="3" t="inlineStr">
+        <is>
+          <t>lights/sun</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="45" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -6289,6 +6342,7 @@
         </is>
       </c>
       <c r="AG42" s="3" t="inlineStr"/>
+      <c r="AH42" s="3" t="inlineStr"/>
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -6347,7 +6401,7 @@
       <c r="N43" s="3" t="inlineStr"/>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar</t>
+          <t>event/state</t>
         </is>
       </c>
       <c r="P43" s="3" t="inlineStr">
@@ -6382,7 +6436,11 @@
       </c>
       <c r="V43" s="3" t="inlineStr"/>
       <c r="W43" s="3" t="inlineStr"/>
-      <c r="X43" s="3" t="inlineStr"/>
+      <c r="X43" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y43" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6408,6 +6466,7 @@
         </is>
       </c>
       <c r="AG43" s="3" t="inlineStr"/>
+      <c r="AH43" s="3" t="inlineStr"/>
     </row>
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
@@ -6527,6 +6586,7 @@
         </is>
       </c>
       <c r="AG44" s="3" t="inlineStr"/>
+      <c r="AH44" s="3" t="inlineStr"/>
     </row>
     <row r="45" ht="45" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
@@ -6646,6 +6706,7 @@
         </is>
       </c>
       <c r="AG45" s="3" t="inlineStr"/>
+      <c r="AH45" s="3" t="inlineStr"/>
     </row>
     <row r="46" ht="45" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
@@ -6765,6 +6826,7 @@
         </is>
       </c>
       <c r="AG46" s="3" t="inlineStr"/>
+      <c r="AH46" s="3" t="inlineStr"/>
     </row>
     <row r="47" ht="45" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
@@ -6884,6 +6946,7 @@
         </is>
       </c>
       <c r="AG47" s="3" t="inlineStr"/>
+      <c r="AH47" s="3" t="inlineStr"/>
     </row>
     <row r="48" ht="45" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
@@ -7003,6 +7066,7 @@
         </is>
       </c>
       <c r="AG48" s="3" t="inlineStr"/>
+      <c r="AH48" s="3" t="inlineStr"/>
     </row>
     <row r="49" ht="45" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
@@ -7122,6 +7186,7 @@
         </is>
       </c>
       <c r="AG49" s="3" t="inlineStr"/>
+      <c r="AH49" s="3" t="inlineStr"/>
     </row>
     <row r="50" ht="45" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
@@ -7241,6 +7306,7 @@
         </is>
       </c>
       <c r="AG50" s="3" t="inlineStr"/>
+      <c r="AH50" s="3" t="inlineStr"/>
     </row>
     <row r="51" ht="45" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -7299,7 +7365,7 @@
       <c r="N51" s="3" t="inlineStr"/>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar</t>
+          <t>clock/calendar</t>
         </is>
       </c>
       <c r="P51" s="3" t="inlineStr">
@@ -7334,7 +7400,11 @@
       </c>
       <c r="V51" s="3" t="inlineStr"/>
       <c r="W51" s="3" t="inlineStr"/>
-      <c r="X51" s="3" t="inlineStr"/>
+      <c r="X51" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y51" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7360,6 +7430,7 @@
         </is>
       </c>
       <c r="AG51" s="3" t="inlineStr"/>
+      <c r="AH51" s="3" t="inlineStr"/>
     </row>
     <row r="52" ht="45" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
@@ -7483,6 +7554,7 @@
         </is>
       </c>
       <c r="AG52" s="3" t="inlineStr"/>
+      <c r="AH52" s="3" t="inlineStr"/>
     </row>
     <row r="53" ht="45" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -7606,6 +7678,7 @@
         </is>
       </c>
       <c r="AG53" s="3" t="inlineStr"/>
+      <c r="AH53" s="3" t="inlineStr"/>
     </row>
     <row r="54" ht="45" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -7729,6 +7802,7 @@
         </is>
       </c>
       <c r="AG54" s="3" t="inlineStr"/>
+      <c r="AH54" s="3" t="inlineStr"/>
     </row>
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -7848,6 +7922,7 @@
         </is>
       </c>
       <c r="AG55" s="3" t="inlineStr"/>
+      <c r="AH55" s="3" t="inlineStr"/>
     </row>
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
@@ -7967,6 +8042,7 @@
         </is>
       </c>
       <c r="AG56" s="3" t="inlineStr"/>
+      <c r="AH56" s="3" t="inlineStr"/>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
@@ -8025,7 +8101,7 @@
       <c r="N57" s="3" t="inlineStr"/>
       <c r="O57" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar</t>
+          <t>event/state</t>
         </is>
       </c>
       <c r="P57" s="3" t="inlineStr">
@@ -8060,7 +8136,11 @@
       </c>
       <c r="V57" s="3" t="inlineStr"/>
       <c r="W57" s="3" t="inlineStr"/>
-      <c r="X57" s="3" t="inlineStr"/>
+      <c r="X57" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y57" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8086,6 +8166,7 @@
         </is>
       </c>
       <c r="AG57" s="3" t="inlineStr"/>
+      <c r="AH57" s="3" t="inlineStr"/>
     </row>
     <row r="58" ht="45" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -8205,6 +8286,7 @@
         </is>
       </c>
       <c r="AG58" s="3" t="inlineStr"/>
+      <c r="AH58" s="3" t="inlineStr"/>
     </row>
     <row r="59" ht="45" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
@@ -8263,12 +8345,12 @@
       <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>event/state</t>
+          <t>event/state; clock/calendar</t>
         </is>
       </c>
       <c r="P59" s="3" t="inlineStr">
         <is>
-          <t>delay/order</t>
+          <t>immediate/unspecified</t>
         </is>
       </c>
       <c r="Q59" s="3" t="inlineStr">
@@ -8298,7 +8380,11 @@
       </c>
       <c r="V59" s="3" t="inlineStr"/>
       <c r="W59" s="3" t="inlineStr"/>
-      <c r="X59" s="3" t="inlineStr"/>
+      <c r="X59" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9</t>
+        </is>
+      </c>
       <c r="Y59" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8324,6 +8410,7 @@
         </is>
       </c>
       <c r="AG59" s="3" t="inlineStr"/>
+      <c r="AH59" s="3" t="inlineStr"/>
     </row>
     <row r="60" ht="45" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
@@ -8443,6 +8530,7 @@
         </is>
       </c>
       <c r="AG60" s="3" t="inlineStr"/>
+      <c r="AH60" s="3" t="inlineStr"/>
     </row>
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
@@ -8562,6 +8650,7 @@
         </is>
       </c>
       <c r="AG61" s="3" t="inlineStr"/>
+      <c r="AH61" s="3" t="inlineStr"/>
     </row>
     <row r="62" ht="45" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
@@ -8687,6 +8776,7 @@
         </is>
       </c>
       <c r="AG62" s="3" t="inlineStr"/>
+      <c r="AH62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -8806,6 +8896,7 @@
         </is>
       </c>
       <c r="AG63" s="3" t="inlineStr"/>
+      <c r="AH63" s="3" t="inlineStr"/>
     </row>
     <row r="64" ht="45" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
@@ -8925,6 +9016,7 @@
         </is>
       </c>
       <c r="AG64" s="3" t="inlineStr"/>
+      <c r="AH64" s="3" t="inlineStr"/>
     </row>
     <row r="65" ht="45" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -9044,6 +9136,7 @@
         </is>
       </c>
       <c r="AG65" s="3" t="inlineStr"/>
+      <c r="AH65" s="3" t="inlineStr"/>
     </row>
     <row r="66" ht="45" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
@@ -9163,6 +9256,7 @@
         </is>
       </c>
       <c r="AG66" s="3" t="inlineStr"/>
+      <c r="AH66" s="3" t="inlineStr"/>
     </row>
     <row r="67" ht="45" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
@@ -9282,6 +9376,7 @@
         </is>
       </c>
       <c r="AG67" s="3" t="inlineStr"/>
+      <c r="AH67" s="3" t="inlineStr"/>
     </row>
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
@@ -9337,11 +9432,7 @@
         </is>
       </c>
       <c r="M68" s="3" t="inlineStr"/>
-      <c r="N68" s="3" t="inlineStr">
-        <is>
-          <t>motion-light</t>
-        </is>
-      </c>
+      <c r="N68" s="3" t="inlineStr"/>
       <c r="O68" s="3" t="inlineStr">
         <is>
           <t>event/state</t>
@@ -9405,6 +9496,11 @@
         </is>
       </c>
       <c r="AG68" s="3" t="inlineStr"/>
+      <c r="AH68" s="3" t="inlineStr">
+        <is>
+          <t>motion-light</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="45" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
@@ -9460,11 +9556,7 @@
         </is>
       </c>
       <c r="M69" s="3" t="inlineStr"/>
-      <c r="N69" s="3" t="inlineStr">
-        <is>
-          <t>motion-light</t>
-        </is>
-      </c>
+      <c r="N69" s="3" t="inlineStr"/>
       <c r="O69" s="3" t="inlineStr">
         <is>
           <t>event/state</t>
@@ -9528,6 +9620,11 @@
         </is>
       </c>
       <c r="AG69" s="3" t="inlineStr"/>
+      <c r="AH69" s="3" t="inlineStr">
+        <is>
+          <t>motion-light</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
@@ -9586,7 +9683,7 @@
       <c r="N70" s="3" t="inlineStr"/>
       <c r="O70" s="3" t="inlineStr">
         <is>
-          <t>clock/calendar</t>
+          <t>event/state</t>
         </is>
       </c>
       <c r="P70" s="3" t="inlineStr">
@@ -9621,7 +9718,11 @@
       </c>
       <c r="V70" s="3" t="inlineStr"/>
       <c r="W70" s="3" t="inlineStr"/>
-      <c r="X70" s="3" t="inlineStr"/>
+      <c r="X70" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y70" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9647,6 +9748,7 @@
         </is>
       </c>
       <c r="AG70" s="3" t="inlineStr"/>
+      <c r="AH70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -9766,6 +9868,7 @@
         </is>
       </c>
       <c r="AG71" s="3" t="inlineStr"/>
+      <c r="AH71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="45" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
@@ -9824,7 +9927,7 @@
       <c r="N72" s="3" t="inlineStr"/>
       <c r="O72" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar; manual</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="P72" s="3" t="inlineStr">
@@ -9859,7 +9962,11 @@
       </c>
       <c r="V72" s="3" t="inlineStr"/>
       <c r="W72" s="3" t="inlineStr"/>
-      <c r="X72" s="3" t="inlineStr"/>
+      <c r="X72" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y72" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9891,6 +9998,7 @@
         </is>
       </c>
       <c r="AG72" s="3" t="inlineStr"/>
+      <c r="AH72" s="3" t="inlineStr"/>
     </row>
     <row r="73" ht="45" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
@@ -9949,12 +10057,12 @@
       <c r="N73" s="3" t="inlineStr"/>
       <c r="O73" s="3" t="inlineStr">
         <is>
-          <t>event/state</t>
+          <t>event/state; clock/calendar</t>
         </is>
       </c>
       <c r="P73" s="3" t="inlineStr">
         <is>
-          <t>delay/order</t>
+          <t>immediate/unspecified</t>
         </is>
       </c>
       <c r="Q73" s="3" t="inlineStr">
@@ -9984,7 +10092,11 @@
       </c>
       <c r="V73" s="3" t="inlineStr"/>
       <c r="W73" s="3" t="inlineStr"/>
-      <c r="X73" s="3" t="inlineStr"/>
+      <c r="X73" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9</t>
+        </is>
+      </c>
       <c r="Y73" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10010,6 +10122,7 @@
         </is>
       </c>
       <c r="AG73" s="3" t="inlineStr"/>
+      <c r="AH73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="45" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
@@ -10088,7 +10201,7 @@
       </c>
       <c r="S74" s="3" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>single</t>
         </is>
       </c>
       <c r="T74" s="3" t="inlineStr">
@@ -10129,6 +10242,7 @@
         </is>
       </c>
       <c r="AG74" s="3" t="inlineStr"/>
+      <c r="AH74" s="3" t="inlineStr"/>
     </row>
     <row r="75" ht="45" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
@@ -10248,6 +10362,7 @@
         </is>
       </c>
       <c r="AG75" s="3" t="inlineStr"/>
+      <c r="AH75" s="3" t="inlineStr"/>
     </row>
     <row r="76" ht="45" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
@@ -10367,6 +10482,7 @@
         </is>
       </c>
       <c r="AG76" s="3" t="inlineStr"/>
+      <c r="AH76" s="3" t="inlineStr"/>
     </row>
     <row r="77" ht="45" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
@@ -10486,6 +10602,7 @@
         </is>
       </c>
       <c r="AG77" s="3" t="inlineStr"/>
+      <c r="AH77" s="3" t="inlineStr"/>
     </row>
     <row r="78" ht="45" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
@@ -10605,6 +10722,7 @@
         </is>
       </c>
       <c r="AG78" s="3" t="inlineStr"/>
+      <c r="AH78" s="3" t="inlineStr"/>
     </row>
     <row r="79" ht="45" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
@@ -10724,6 +10842,7 @@
         </is>
       </c>
       <c r="AG79" s="3" t="inlineStr"/>
+      <c r="AH79" s="3" t="inlineStr"/>
     </row>
     <row r="80" ht="45" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
@@ -10843,6 +10962,7 @@
         </is>
       </c>
       <c r="AG80" s="3" t="inlineStr"/>
+      <c r="AH80" s="3" t="inlineStr"/>
     </row>
     <row r="81" ht="45" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
@@ -10962,6 +11082,7 @@
         </is>
       </c>
       <c r="AG81" s="3" t="inlineStr"/>
+      <c r="AH81" s="3" t="inlineStr"/>
     </row>
     <row r="82" ht="45" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
@@ -11081,6 +11202,7 @@
         </is>
       </c>
       <c r="AG82" s="3" t="inlineStr"/>
+      <c r="AH82" s="3" t="inlineStr"/>
     </row>
     <row r="83" ht="45" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
@@ -11159,7 +11281,7 @@
       </c>
       <c r="S83" s="3" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>single</t>
         </is>
       </c>
       <c r="T83" s="3" t="inlineStr">
@@ -11200,6 +11322,7 @@
         </is>
       </c>
       <c r="AG83" s="3" t="inlineStr"/>
+      <c r="AH83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="45" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
@@ -11327,6 +11450,7 @@
         </is>
       </c>
       <c r="AG84" s="3" t="inlineStr"/>
+      <c r="AH84" s="3" t="inlineStr"/>
     </row>
     <row r="85" ht="45" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
@@ -11446,6 +11570,7 @@
         </is>
       </c>
       <c r="AG85" s="3" t="inlineStr"/>
+      <c r="AH85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="45" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
@@ -11565,6 +11690,7 @@
         </is>
       </c>
       <c r="AG86" s="3" t="inlineStr"/>
+      <c r="AH86" s="3" t="inlineStr"/>
     </row>
     <row r="87" ht="45" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
@@ -11690,6 +11816,7 @@
         </is>
       </c>
       <c r="AG87" s="3" t="inlineStr"/>
+      <c r="AH87" s="3" t="inlineStr"/>
     </row>
     <row r="88" ht="45" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
@@ -11745,11 +11872,7 @@
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr"/>
-      <c r="N88" s="3" t="inlineStr">
-        <is>
-          <t>timed-on</t>
-        </is>
-      </c>
+      <c r="N88" s="3" t="inlineStr"/>
       <c r="O88" s="3" t="inlineStr">
         <is>
           <t>event/state; manual</t>
@@ -11813,6 +11936,11 @@
         </is>
       </c>
       <c r="AG88" s="3" t="inlineStr"/>
+      <c r="AH88" s="3" t="inlineStr">
+        <is>
+          <t>timed-on</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="45" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
@@ -11876,7 +12004,7 @@
       </c>
       <c r="P89" s="3" t="inlineStr">
         <is>
-          <t>duration/window</t>
+          <t>immediate/unspecified</t>
         </is>
       </c>
       <c r="Q89" s="3" t="inlineStr">
@@ -11906,7 +12034,11 @@
       </c>
       <c r="V89" s="3" t="inlineStr"/>
       <c r="W89" s="3" t="inlineStr"/>
-      <c r="X89" s="3" t="inlineStr"/>
+      <c r="X89" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9</t>
+        </is>
+      </c>
       <c r="Y89" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11932,6 +12064,7 @@
         </is>
       </c>
       <c r="AG89" s="3" t="inlineStr"/>
+      <c r="AH89" s="3" t="inlineStr"/>
     </row>
     <row r="90" ht="45" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
@@ -12051,6 +12184,7 @@
         </is>
       </c>
       <c r="AG90" s="3" t="inlineStr"/>
+      <c r="AH90" s="3" t="inlineStr"/>
     </row>
     <row r="91" ht="45" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
@@ -12106,11 +12240,7 @@
         </is>
       </c>
       <c r="M91" s="3" t="inlineStr"/>
-      <c r="N91" s="3" t="inlineStr">
-        <is>
-          <t>timed-on</t>
-        </is>
-      </c>
+      <c r="N91" s="3" t="inlineStr"/>
       <c r="O91" s="3" t="inlineStr">
         <is>
           <t>unspecified</t>
@@ -12174,6 +12304,11 @@
         </is>
       </c>
       <c r="AG91" s="3" t="inlineStr"/>
+      <c r="AH91" s="3" t="inlineStr">
+        <is>
+          <t>timed-on</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="45" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
@@ -12230,7 +12365,7 @@
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>The source leaves a behavior-defining choice unresolved.</t>
+          <t>The source does not state the content of the joint condition over the valve positions.</t>
         </is>
       </c>
       <c r="N92" s="3" t="inlineStr"/>
@@ -12301,6 +12436,7 @@
         </is>
       </c>
       <c r="AG92" s="3" t="inlineStr"/>
+      <c r="AH92" s="3" t="inlineStr"/>
     </row>
     <row r="93" ht="45" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
@@ -12356,11 +12492,7 @@
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr"/>
-      <c r="N93" s="3" t="inlineStr">
-        <is>
-          <t>parallel-flow</t>
-        </is>
-      </c>
+      <c r="N93" s="3" t="inlineStr"/>
       <c r="O93" s="3" t="inlineStr">
         <is>
           <t>event/state</t>
@@ -12430,6 +12562,11 @@
         </is>
       </c>
       <c r="AG93" s="3" t="inlineStr"/>
+      <c r="AH93" s="3" t="inlineStr">
+        <is>
+          <t>parallel-flow</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="45" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
@@ -12485,14 +12622,10 @@
         </is>
       </c>
       <c r="M94" s="3" t="inlineStr"/>
-      <c r="N94" s="3" t="inlineStr">
-        <is>
-          <t>parallel-flow</t>
-        </is>
-      </c>
+      <c r="N94" s="3" t="inlineStr"/>
       <c r="O94" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar</t>
+          <t>event/state</t>
         </is>
       </c>
       <c r="P94" s="3" t="inlineStr">
@@ -12553,6 +12686,11 @@
         </is>
       </c>
       <c r="AG94" s="3" t="inlineStr"/>
+      <c r="AH94" s="3" t="inlineStr">
+        <is>
+          <t>parallel-flow</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="45" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
@@ -12608,11 +12746,7 @@
         </is>
       </c>
       <c r="M95" s="3" t="inlineStr"/>
-      <c r="N95" s="3" t="inlineStr">
-        <is>
-          <t>parallel-flow</t>
-        </is>
-      </c>
+      <c r="N95" s="3" t="inlineStr"/>
       <c r="O95" s="3" t="inlineStr">
         <is>
           <t>unspecified</t>
@@ -12676,6 +12810,11 @@
         </is>
       </c>
       <c r="AG95" s="3" t="inlineStr"/>
+      <c r="AH95" s="3" t="inlineStr">
+        <is>
+          <t>parallel-flow</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="45" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
@@ -12727,7 +12866,7 @@
       <c r="K96" s="3" t="inlineStr"/>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>AMBIGUOUS</t>
+          <t>IN_SCOPE</t>
         </is>
       </c>
       <c r="M96" s="3" t="inlineStr">
@@ -12792,11 +12931,7 @@
           <t>Primary internal accumulation/average boundary probe; semantics must be fixed first.</t>
         </is>
       </c>
-      <c r="AC96" s="3" t="inlineStr">
-        <is>
-          <t>Needs a case-specific interpretation question before any depth encoding.</t>
-        </is>
-      </c>
+      <c r="AC96" s="3" t="inlineStr"/>
       <c r="AD96" s="3" t="inlineStr"/>
       <c r="AE96" s="3" t="inlineStr">
         <is>
@@ -12808,7 +12943,12 @@
           <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
-      <c r="AG96" s="3" t="inlineStr"/>
+      <c r="AG96" s="3" t="inlineStr">
+        <is>
+          <t>Author interpretation: read pH and chlorine at 10:00, 11:00, 12:00, 13:00 and 14:00 (five samples) and report each mean at 15:00.</t>
+        </is>
+      </c>
+      <c r="AH96" s="3" t="inlineStr"/>
     </row>
     <row r="97" ht="45" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
@@ -12928,6 +13068,7 @@
         </is>
       </c>
       <c r="AG97" s="3" t="inlineStr"/>
+      <c r="AH97" s="3" t="inlineStr"/>
     </row>
     <row r="98" ht="45" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
@@ -12983,14 +13124,10 @@
         </is>
       </c>
       <c r="M98" s="3" t="inlineStr"/>
-      <c r="N98" s="3" t="inlineStr">
-        <is>
-          <t>parallel-flow</t>
-        </is>
-      </c>
+      <c r="N98" s="3" t="inlineStr"/>
       <c r="O98" s="3" t="inlineStr">
         <is>
-          <t>clock/calendar; manual</t>
+          <t>event/state</t>
         </is>
       </c>
       <c r="P98" s="3" t="inlineStr">
@@ -13000,7 +13137,7 @@
       </c>
       <c r="Q98" s="3" t="inlineStr">
         <is>
-          <t>sequence/composition; parallel</t>
+          <t>sequence/composition; guard/branch; parallel</t>
         </is>
       </c>
       <c r="R98" s="3" t="inlineStr">
@@ -13051,6 +13188,11 @@
         </is>
       </c>
       <c r="AG98" s="3" t="inlineStr"/>
+      <c r="AH98" s="3" t="inlineStr">
+        <is>
+          <t>parallel-flow</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="45" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
@@ -13170,6 +13312,7 @@
         </is>
       </c>
       <c r="AG99" s="3" t="inlineStr"/>
+      <c r="AH99" s="3" t="inlineStr"/>
     </row>
     <row r="100" ht="45" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
@@ -13295,6 +13438,7 @@
         </is>
       </c>
       <c r="AG100" s="3" t="inlineStr"/>
+      <c r="AH100" s="3" t="inlineStr"/>
     </row>
     <row r="101" ht="45" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
@@ -13373,7 +13517,7 @@
       </c>
       <c r="S101" s="3" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>single</t>
         </is>
       </c>
       <c r="T101" s="3" t="inlineStr">
@@ -13414,9 +13558,10 @@
         </is>
       </c>
       <c r="AG101" s="3" t="inlineStr"/>
+      <c r="AH101" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG101"/>
+  <autoFilter ref="A1:AH101"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -13533,7 +13678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG21"/>
+  <dimension ref="A1:AH21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13569,6 +13714,7 @@
     <col width="24" customWidth="1" min="31" max="31"/>
     <col width="24" customWidth="1" min="32" max="32"/>
     <col width="42" customWidth="1" min="33" max="33"/>
+    <col width="15" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13735,6 +13881,11 @@
       <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>topic_family</t>
         </is>
       </c>
     </row>
@@ -13864,6 +14015,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -13991,6 +14143,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -14118,6 +14271,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -14245,6 +14399,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -14372,6 +14527,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -14499,6 +14655,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -14626,6 +14783,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -14753,6 +14911,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -14880,6 +15039,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -15007,6 +15167,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -15134,6 +15295,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -15261,6 +15423,7 @@
           <t>Stage A selection was a work-unit decision; no statistical sample-size rationale is claimed.</t>
         </is>
       </c>
+      <c r="AH13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -15316,11 +15479,7 @@
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>parallel-flow</t>
-        </is>
-      </c>
+      <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
           <t>event/state</t>
@@ -15390,6 +15549,11 @@
         </is>
       </c>
       <c r="AG14" s="3" t="inlineStr"/>
+      <c r="AH14" s="3" t="inlineStr">
+        <is>
+          <t>parallel-flow</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -15441,7 +15605,7 @@
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>AMBIGUOUS</t>
+          <t>IN_SCOPE</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -15506,11 +15670,7 @@
           <t>Primary internal accumulation/average boundary probe; semantics must be fixed first.</t>
         </is>
       </c>
-      <c r="AC15" s="3" t="inlineStr">
-        <is>
-          <t>Needs a case-specific interpretation question before any depth encoding.</t>
-        </is>
-      </c>
+      <c r="AC15" s="3" t="inlineStr"/>
       <c r="AD15" s="3" t="inlineStr"/>
       <c r="AE15" s="3" t="inlineStr">
         <is>
@@ -15522,7 +15682,12 @@
           <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
         </is>
       </c>
-      <c r="AG15" s="3" t="inlineStr"/>
+      <c r="AG15" s="3" t="inlineStr">
+        <is>
+          <t>Author interpretation: read pH and chlorine at 10:00, 11:00, 12:00, 13:00 and 14:00 (five samples) and report each mean at 15:00.</t>
+        </is>
+      </c>
+      <c r="AH15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -15648,6 +15813,7 @@
         </is>
       </c>
       <c r="AG16" s="3" t="inlineStr"/>
+      <c r="AH16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -15773,6 +15939,7 @@
         </is>
       </c>
       <c r="AG17" s="3" t="inlineStr"/>
+      <c r="AH17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -15906,6 +16073,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH18" s="3" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -16039,6 +16207,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH19" s="3" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -16097,7 +16266,7 @@
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>event/state; clock/calendar; manual</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="P20" s="3" t="inlineStr">
@@ -16132,7 +16301,11 @@
       </c>
       <c r="V20" s="3" t="inlineStr"/>
       <c r="W20" s="3" t="inlineStr"/>
-      <c r="X20" s="3" t="inlineStr"/>
+      <c r="X20" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -16164,6 +16337,7 @@
         </is>
       </c>
       <c r="AG20" s="3" t="inlineStr"/>
+      <c r="AH20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -16289,9 +16463,10 @@
         </is>
       </c>
       <c r="AG21" s="3" t="inlineStr"/>
+      <c r="AH21" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG21"/>
+  <autoFilter ref="A1:AH21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -16328,7 +16503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG10"/>
+  <dimension ref="A1:AH9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16351,7 +16526,7 @@
     <col width="24" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
@@ -16364,6 +16539,7 @@
     <col width="24" customWidth="1" min="31" max="31"/>
     <col width="24" customWidth="1" min="32" max="32"/>
     <col width="42" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16532,6 +16708,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>topic_family</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -16667,6 +16848,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -16802,6 +16984,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -16937,11 +17120,12 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>E1-031</t>
+          <t>E1-027</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -16972,7 +17156,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Result sheet, Excel row 48, column CF (header 10_Q25, statement 10)</t>
+          <t>Result sheet, Excel row 21, column AR (header 2_Q25, statement 2)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -16982,28 +17166,28 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>The Smart TV in the children's room should never turn on whenever the toothbrush has not been used at least twice that day</t>
+          <t>my outdoor lights should always be on between 7 and 12 pm</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>ReleaseData=Yes; saw_examples=yes; exception_response=none</t>
+          <t>ReleaseData=Yes; saw_examples=yes; exception_response=possibly if I am out of town then the lights wouldn't need to be on.</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>UNMATCHED</t>
+          <t>AMBIGUOUS</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Clear daily-count requirement, but the current service catalog does not expose the required history/count value.</t>
+          <t>The clock meaning of 'between 7 and 12 pm' is unclear; the original text is kept without normalization.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>event/state</t>
+          <t>clock/calendar</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -17013,17 +17197,17 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>straight-line/unspecified</t>
+          <t>sequence/composition</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>count/aggregate</t>
+          <t>none/unspecified</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
@@ -17033,7 +17217,7 @@
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>R1, R8</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr"/>
@@ -17051,12 +17235,12 @@
       </c>
       <c r="AA5" s="3" t="inlineStr"/>
       <c r="AB5" s="3" t="inlineStr"/>
-      <c r="AC5" s="3" t="inlineStr"/>
-      <c r="AD5" s="3" t="inlineStr">
-        <is>
-          <t>Becomes expressible if a history/count service supplies the daily count; this is not evidence of an IR-language boundary.</t>
-        </is>
-      </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>Which time range 'between 7 and 12 pm' denotes.</t>
+        </is>
+      </c>
+      <c r="AD5" s="3" t="inlineStr"/>
       <c r="AE5" s="3" t="inlineStr">
         <is>
           <t>VERBATIM_PUBLIC_STUDY_DATA</t>
@@ -17072,6 +17256,7 @@
           <t>Original spelling preserved.</t>
         </is>
       </c>
+      <c r="AH5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -17195,6 +17380,7 @@
         </is>
       </c>
       <c r="AG6" s="3" t="inlineStr"/>
+      <c r="AH6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -17318,6 +17504,7 @@
         </is>
       </c>
       <c r="AG7" s="3" t="inlineStr"/>
+      <c r="AH7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -17445,6 +17632,7 @@
         </is>
       </c>
       <c r="AG8" s="3" t="inlineStr"/>
+      <c r="AH8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -17501,7 +17689,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>The source leaves a behavior-defining choice unresolved.</t>
+          <t>The source does not state the content of the joint condition over the valve positions.</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr"/>
@@ -17572,142 +17760,10 @@
         </is>
       </c>
       <c r="AG9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>E1-095</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>community</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>user-authored naturalistic</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Home Assistant Community thread 654561: Getting an average reading of a sensor during certain hours</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>https://community.home-assistant.io/t/getting-an-average-reading-of-a-sensor-during-certain-hours/654561</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>opening post (created 2023-12-12 UTC)</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Calculate the average pH and chlorine levels between 10:00 and 15:00 and report those readings daily.</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>AMBIGUOUS</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>The source leaves a behavior-defining choice unresolved.</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr"/>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>clock/calendar</t>
-        </is>
-      </c>
-      <c r="P10" s="3" t="inlineStr">
-        <is>
-          <t>periodic/count</t>
-        </is>
-      </c>
-      <c r="Q10" s="3" t="inlineStr">
-        <is>
-          <t>sequence/composition</t>
-        </is>
-      </c>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>count/aggregate</t>
-        </is>
-      </c>
-      <c r="S10" s="3" t="inlineStr">
-        <is>
-          <t>multiple</t>
-        </is>
-      </c>
-      <c r="T10" s="3" t="inlineStr">
-        <is>
-          <t>recurring</t>
-        </is>
-      </c>
-      <c r="U10" s="3" t="inlineStr">
-        <is>
-          <t>R5, R9, L-ACCUM</t>
-        </is>
-      </c>
-      <c r="V10" s="3" t="inlineStr"/>
-      <c r="W10" s="3" t="inlineStr"/>
-      <c r="X10" s="3" t="inlineStr"/>
-      <c r="Y10" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="Z10" s="3" t="inlineStr">
-        <is>
-          <t>proposed_depth_addition</t>
-        </is>
-      </c>
-      <c r="AA10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB10" s="3" t="inlineStr">
-        <is>
-          <t>Primary internal accumulation/average boundary probe; semantics must be fixed first.</t>
-        </is>
-      </c>
-      <c r="AC10" s="3" t="inlineStr">
-        <is>
-          <t>Needs a case-specific interpretation question before any depth encoding.</t>
-        </is>
-      </c>
-      <c r="AD10" s="3" t="inlineStr"/>
-      <c r="AE10" s="3" t="inlineStr">
-        <is>
-          <t>RESEARCHER_NORMALIZATION_OF_STATED_BEHAVIOR</t>
-        </is>
-      </c>
-      <c r="AF10" s="3" t="inlineStr">
-        <is>
-          <t>SERVER_CHECKED_2026-09-13; CORRECTED</t>
-        </is>
-      </c>
-      <c r="AG10" s="3" t="inlineStr"/>
+      <c r="AH9" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG10"/>
+  <autoFilter ref="A1:AH9"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
@@ -17717,12 +17773,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -23300,7 +23355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23406,34 +23461,70 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>text_form</t>
+          <t>rb_adjudicated</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Whether text is verbatim, source-extracted, or researcher-normalized.</t>
+          <t>The author's R/B labels (single author; column name kept for compatibility).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>completed_seed</t>
+          <t>duplicate_family</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>One of the existing 12 depth cases.</t>
+          <t>Verified duplicate group under protocol §2; empty for all 100 (no retained duplicate).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>topic_family</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Similar-topic group; not a duplicate mark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>text_form</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Whether text is verbatim, source-extracted, or researcher-normalized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>completed_seed</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>One of the existing 12 depth cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>One of eight new candidates; freeze before encoding.</t>
         </is>

</xml_diff>

<commit_message>
E1 breadth: apply author R/B coding (92 IN_SCOPE rows)
- rb_adjudicated: Stage A codes for the 12 seeds, 17 author exception labels,
  author-approved preliminary codes for the other 63 IN_SCOPE rows, N/A for the
  6 AMBIGUOUS and 2 OUT_OF_SCOPE rows; rb_preliminary kept for provenance
- L-ACCUM removed from final codes (E1-095: R5, R8, R9)
- protocol §5: single-author screening of 100, R/B denominator 92, no kappa
- record audit/AUTHOR_RB_CODING_2026-09-13.md, change log (92), workbook rebuilt
- build_workbook.py: read CSVs with keep_default_na=False so N/A is kept

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPrygyUUKfHFM8zKEvmbin
</commit_message>
<xml_diff>
--- a/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
+++ b/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e1-corpus-v0.2-author-screened</t>
+          <t>e1-corpus-v0.3-author-coded</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>• Screening status is the author's manual screening (2026-09-13); no retained duplicate. No second coder or kappa is used. rb_preliminary is triage only; rb_adjudicated holds the author's R/B labels and is incomplete.</t>
+          <t>• Screening status is the author's manual screening (2026-09-13); no retained duplicate. No second coder or kappa is used. rb_preliminary is triage only; rb_adjudicated holds the author's final R/B codes for the 92 IN_SCOPE rows (N/A for the other 8); R/B counts use denominator 92.</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
@@ -1176,7 +1176,11 @@
       </c>
       <c r="V2" s="3" t="inlineStr"/>
       <c r="W2" s="3" t="inlineStr"/>
-      <c r="X2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3, R7, B1</t>
+        </is>
+      </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1304,7 +1308,11 @@
       </c>
       <c r="V3" s="3" t="inlineStr"/>
       <c r="W3" s="3" t="inlineStr"/>
-      <c r="X3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2</t>
+        </is>
+      </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1432,7 +1440,11 @@
       </c>
       <c r="V4" s="3" t="inlineStr"/>
       <c r="W4" s="3" t="inlineStr"/>
-      <c r="X4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>R9, R2</t>
+        </is>
+      </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1560,7 +1572,11 @@
       </c>
       <c r="V5" s="3" t="inlineStr"/>
       <c r="W5" s="3" t="inlineStr"/>
-      <c r="X5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>R3, R7</t>
+        </is>
+      </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1688,7 +1704,11 @@
       </c>
       <c r="V6" s="3" t="inlineStr"/>
       <c r="W6" s="3" t="inlineStr"/>
-      <c r="X6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>R9, R3, R5, R8, B5, B1</t>
+        </is>
+      </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1816,7 +1836,11 @@
       </c>
       <c r="V7" s="3" t="inlineStr"/>
       <c r="W7" s="3" t="inlineStr"/>
-      <c r="X7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>R1, R4</t>
+        </is>
+      </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1944,7 +1968,11 @@
       </c>
       <c r="V8" s="3" t="inlineStr"/>
       <c r="W8" s="3" t="inlineStr"/>
-      <c r="X8" s="3" t="inlineStr"/>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>R1, B2</t>
+        </is>
+      </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2072,7 +2100,11 @@
       </c>
       <c r="V9" s="3" t="inlineStr"/>
       <c r="W9" s="3" t="inlineStr"/>
-      <c r="X9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>R4, R7, R9</t>
+        </is>
+      </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2200,7 +2232,11 @@
       </c>
       <c r="V10" s="3" t="inlineStr"/>
       <c r="W10" s="3" t="inlineStr"/>
-      <c r="X10" s="3" t="inlineStr"/>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
+          <t>R9, R6</t>
+        </is>
+      </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2328,7 +2364,11 @@
       </c>
       <c r="V11" s="3" t="inlineStr"/>
       <c r="W11" s="3" t="inlineStr"/>
-      <c r="X11" s="3" t="inlineStr"/>
+      <c r="X11" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9, R2</t>
+        </is>
+      </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2456,7 +2496,11 @@
       </c>
       <c r="V12" s="3" t="inlineStr"/>
       <c r="W12" s="3" t="inlineStr"/>
-      <c r="X12" s="3" t="inlineStr"/>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>R10, R9</t>
+        </is>
+      </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2584,7 +2628,11 @@
       </c>
       <c r="V13" s="3" t="inlineStr"/>
       <c r="W13" s="3" t="inlineStr"/>
-      <c r="X13" s="3" t="inlineStr"/>
+      <c r="X13" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, B1</t>
+        </is>
+      </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2712,7 +2760,11 @@
       </c>
       <c r="V14" s="3" t="inlineStr"/>
       <c r="W14" s="3" t="inlineStr"/>
-      <c r="X14" s="3" t="inlineStr"/>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3</t>
+        </is>
+      </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -2840,7 +2892,11 @@
       </c>
       <c r="V15" s="3" t="inlineStr"/>
       <c r="W15" s="3" t="inlineStr"/>
-      <c r="X15" s="3" t="inlineStr"/>
+      <c r="X15" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3</t>
+        </is>
+      </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -2972,7 +3028,11 @@
       </c>
       <c r="V16" s="3" t="inlineStr"/>
       <c r="W16" s="3" t="inlineStr"/>
-      <c r="X16" s="3" t="inlineStr"/>
+      <c r="X16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3104,7 +3164,11 @@
       </c>
       <c r="V17" s="3" t="inlineStr"/>
       <c r="W17" s="3" t="inlineStr"/>
-      <c r="X17" s="3" t="inlineStr"/>
+      <c r="X17" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y17" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3236,7 +3300,11 @@
       </c>
       <c r="V18" s="3" t="inlineStr"/>
       <c r="W18" s="3" t="inlineStr"/>
-      <c r="X18" s="3" t="inlineStr"/>
+      <c r="X18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3372,7 +3440,11 @@
       </c>
       <c r="V19" s="3" t="inlineStr"/>
       <c r="W19" s="3" t="inlineStr"/>
-      <c r="X19" s="3" t="inlineStr"/>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y19" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3504,7 +3576,11 @@
       </c>
       <c r="V20" s="3" t="inlineStr"/>
       <c r="W20" s="3" t="inlineStr"/>
-      <c r="X20" s="3" t="inlineStr"/>
+      <c r="X20" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3632,7 +3708,11 @@
       </c>
       <c r="V21" s="3" t="inlineStr"/>
       <c r="W21" s="3" t="inlineStr"/>
-      <c r="X21" s="3" t="inlineStr"/>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y21" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3760,7 +3840,11 @@
       </c>
       <c r="V22" s="3" t="inlineStr"/>
       <c r="W22" s="3" t="inlineStr"/>
-      <c r="X22" s="3" t="inlineStr"/>
+      <c r="X22" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y22" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -3888,7 +3972,11 @@
       </c>
       <c r="V23" s="3" t="inlineStr"/>
       <c r="W23" s="3" t="inlineStr"/>
-      <c r="X23" s="3" t="inlineStr"/>
+      <c r="X23" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y23" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4016,7 +4104,11 @@
       </c>
       <c r="V24" s="3" t="inlineStr"/>
       <c r="W24" s="3" t="inlineStr"/>
-      <c r="X24" s="3" t="inlineStr"/>
+      <c r="X24" s="3" t="inlineStr">
+        <is>
+          <t>R1, B3</t>
+        </is>
+      </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4144,7 +4236,11 @@
       </c>
       <c r="V25" s="3" t="inlineStr"/>
       <c r="W25" s="3" t="inlineStr"/>
-      <c r="X25" s="3" t="inlineStr"/>
+      <c r="X25" s="3" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
       <c r="Y25" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4272,7 +4368,11 @@
       </c>
       <c r="V26" s="3" t="inlineStr"/>
       <c r="W26" s="3" t="inlineStr"/>
-      <c r="X26" s="3" t="inlineStr"/>
+      <c r="X26" s="3" t="inlineStr">
+        <is>
+          <t>R2, R9</t>
+        </is>
+      </c>
       <c r="Y26" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4400,7 +4500,11 @@
       </c>
       <c r="V27" s="3" t="inlineStr"/>
       <c r="W27" s="3" t="inlineStr"/>
-      <c r="X27" s="3" t="inlineStr"/>
+      <c r="X27" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y27" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4532,7 +4636,11 @@
       </c>
       <c r="V28" s="3" t="inlineStr"/>
       <c r="W28" s="3" t="inlineStr"/>
-      <c r="X28" s="3" t="inlineStr"/>
+      <c r="X28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y28" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4664,7 +4772,11 @@
       </c>
       <c r="V29" s="3" t="inlineStr"/>
       <c r="W29" s="3" t="inlineStr"/>
-      <c r="X29" s="3" t="inlineStr"/>
+      <c r="X29" s="3" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
       <c r="Y29" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4675,8 +4787,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA29" s="3" t="n">
-        <v>5</v>
+      <c r="AA29" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="AB29" s="3" t="inlineStr">
         <is>
@@ -4798,7 +4912,11 @@
       </c>
       <c r="V30" s="3" t="inlineStr"/>
       <c r="W30" s="3" t="inlineStr"/>
-      <c r="X30" s="3" t="inlineStr"/>
+      <c r="X30" s="3" t="inlineStr">
+        <is>
+          <t>R2, B3</t>
+        </is>
+      </c>
       <c r="Y30" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4926,7 +5044,11 @@
       </c>
       <c r="V31" s="3" t="inlineStr"/>
       <c r="W31" s="3" t="inlineStr"/>
-      <c r="X31" s="3" t="inlineStr"/>
+      <c r="X31" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y31" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5054,7 +5176,11 @@
       </c>
       <c r="V32" s="3" t="inlineStr"/>
       <c r="W32" s="3" t="inlineStr"/>
-      <c r="X32" s="3" t="inlineStr"/>
+      <c r="X32" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y32" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5186,7 +5312,11 @@
       </c>
       <c r="V33" s="3" t="inlineStr"/>
       <c r="W33" s="3" t="inlineStr"/>
-      <c r="X33" s="3" t="inlineStr"/>
+      <c r="X33" s="3" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5314,7 +5444,11 @@
       </c>
       <c r="V34" s="3" t="inlineStr"/>
       <c r="W34" s="3" t="inlineStr"/>
-      <c r="X34" s="3" t="inlineStr"/>
+      <c r="X34" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y34" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5442,7 +5576,11 @@
       </c>
       <c r="V35" s="3" t="inlineStr"/>
       <c r="W35" s="3" t="inlineStr"/>
-      <c r="X35" s="3" t="inlineStr"/>
+      <c r="X35" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y35" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5453,8 +5591,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA35" s="3" t="n">
-        <v>6</v>
+      <c r="AA35" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="AB35" s="3" t="inlineStr">
         <is>
@@ -5576,7 +5716,11 @@
       </c>
       <c r="V36" s="3" t="inlineStr"/>
       <c r="W36" s="3" t="inlineStr"/>
-      <c r="X36" s="3" t="inlineStr"/>
+      <c r="X36" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3</t>
+        </is>
+      </c>
       <c r="Y36" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5704,7 +5848,11 @@
       </c>
       <c r="V37" s="3" t="inlineStr"/>
       <c r="W37" s="3" t="inlineStr"/>
-      <c r="X37" s="3" t="inlineStr"/>
+      <c r="X37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y37" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5828,7 +5976,11 @@
       </c>
       <c r="V38" s="3" t="inlineStr"/>
       <c r="W38" s="3" t="inlineStr"/>
-      <c r="X38" s="3" t="inlineStr"/>
+      <c r="X38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y38" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5948,7 +6100,11 @@
       </c>
       <c r="V39" s="3" t="inlineStr"/>
       <c r="W39" s="3" t="inlineStr"/>
-      <c r="X39" s="3" t="inlineStr"/>
+      <c r="X39" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y39" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6068,7 +6224,11 @@
       </c>
       <c r="V40" s="3" t="inlineStr"/>
       <c r="W40" s="3" t="inlineStr"/>
-      <c r="X40" s="3" t="inlineStr"/>
+      <c r="X40" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y40" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6192,7 +6352,11 @@
       </c>
       <c r="V41" s="3" t="inlineStr"/>
       <c r="W41" s="3" t="inlineStr"/>
-      <c r="X41" s="3" t="inlineStr"/>
+      <c r="X41" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, R9</t>
+        </is>
+      </c>
       <c r="Y41" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6316,7 +6480,11 @@
       </c>
       <c r="V42" s="3" t="inlineStr"/>
       <c r="W42" s="3" t="inlineStr"/>
-      <c r="X42" s="3" t="inlineStr"/>
+      <c r="X42" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y42" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6560,7 +6728,11 @@
       </c>
       <c r="V44" s="3" t="inlineStr"/>
       <c r="W44" s="3" t="inlineStr"/>
-      <c r="X44" s="3" t="inlineStr"/>
+      <c r="X44" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y44" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6680,7 +6852,11 @@
       </c>
       <c r="V45" s="3" t="inlineStr"/>
       <c r="W45" s="3" t="inlineStr"/>
-      <c r="X45" s="3" t="inlineStr"/>
+      <c r="X45" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y45" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6800,7 +6976,11 @@
       </c>
       <c r="V46" s="3" t="inlineStr"/>
       <c r="W46" s="3" t="inlineStr"/>
-      <c r="X46" s="3" t="inlineStr"/>
+      <c r="X46" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -6920,7 +7100,11 @@
       </c>
       <c r="V47" s="3" t="inlineStr"/>
       <c r="W47" s="3" t="inlineStr"/>
-      <c r="X47" s="3" t="inlineStr"/>
+      <c r="X47" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y47" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7040,7 +7224,11 @@
       </c>
       <c r="V48" s="3" t="inlineStr"/>
       <c r="W48" s="3" t="inlineStr"/>
-      <c r="X48" s="3" t="inlineStr"/>
+      <c r="X48" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, R9</t>
+        </is>
+      </c>
       <c r="Y48" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7160,7 +7348,11 @@
       </c>
       <c r="V49" s="3" t="inlineStr"/>
       <c r="W49" s="3" t="inlineStr"/>
-      <c r="X49" s="3" t="inlineStr"/>
+      <c r="X49" s="3" t="inlineStr">
+        <is>
+          <t>R5, R6</t>
+        </is>
+      </c>
       <c r="Y49" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7280,7 +7472,11 @@
       </c>
       <c r="V50" s="3" t="inlineStr"/>
       <c r="W50" s="3" t="inlineStr"/>
-      <c r="X50" s="3" t="inlineStr"/>
+      <c r="X50" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, R9</t>
+        </is>
+      </c>
       <c r="Y50" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7524,7 +7720,11 @@
       </c>
       <c r="V52" s="3" t="inlineStr"/>
       <c r="W52" s="3" t="inlineStr"/>
-      <c r="X52" s="3" t="inlineStr"/>
+      <c r="X52" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, R9</t>
+        </is>
+      </c>
       <c r="Y52" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7648,7 +7848,11 @@
       </c>
       <c r="V53" s="3" t="inlineStr"/>
       <c r="W53" s="3" t="inlineStr"/>
-      <c r="X53" s="3" t="inlineStr"/>
+      <c r="X53" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y53" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7772,7 +7976,11 @@
       </c>
       <c r="V54" s="3" t="inlineStr"/>
       <c r="W54" s="3" t="inlineStr"/>
-      <c r="X54" s="3" t="inlineStr"/>
+      <c r="X54" s="3" t="inlineStr">
+        <is>
+          <t>R1, R5, R6, R9</t>
+        </is>
+      </c>
       <c r="Y54" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -7896,7 +8104,11 @@
       </c>
       <c r="V55" s="3" t="inlineStr"/>
       <c r="W55" s="3" t="inlineStr"/>
-      <c r="X55" s="3" t="inlineStr"/>
+      <c r="X55" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y55" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8016,7 +8228,11 @@
       </c>
       <c r="V56" s="3" t="inlineStr"/>
       <c r="W56" s="3" t="inlineStr"/>
-      <c r="X56" s="3" t="inlineStr"/>
+      <c r="X56" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y56" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8260,7 +8476,11 @@
       </c>
       <c r="V58" s="3" t="inlineStr"/>
       <c r="W58" s="3" t="inlineStr"/>
-      <c r="X58" s="3" t="inlineStr"/>
+      <c r="X58" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y58" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8504,7 +8724,11 @@
       </c>
       <c r="V60" s="3" t="inlineStr"/>
       <c r="W60" s="3" t="inlineStr"/>
-      <c r="X60" s="3" t="inlineStr"/>
+      <c r="X60" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y60" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8624,7 +8848,11 @@
       </c>
       <c r="V61" s="3" t="inlineStr"/>
       <c r="W61" s="3" t="inlineStr"/>
-      <c r="X61" s="3" t="inlineStr"/>
+      <c r="X61" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y61" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8744,7 +8972,11 @@
       </c>
       <c r="V62" s="3" t="inlineStr"/>
       <c r="W62" s="3" t="inlineStr"/>
-      <c r="X62" s="3" t="inlineStr"/>
+      <c r="X62" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y62" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8755,8 +8987,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA62" s="3" t="n">
-        <v>8</v>
+      <c r="AA62" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="AB62" s="3" t="inlineStr">
         <is>
@@ -8870,7 +9104,11 @@
       </c>
       <c r="V63" s="3" t="inlineStr"/>
       <c r="W63" s="3" t="inlineStr"/>
-      <c r="X63" s="3" t="inlineStr"/>
+      <c r="X63" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6</t>
+        </is>
+      </c>
       <c r="Y63" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -8990,7 +9228,11 @@
       </c>
       <c r="V64" s="3" t="inlineStr"/>
       <c r="W64" s="3" t="inlineStr"/>
-      <c r="X64" s="3" t="inlineStr"/>
+      <c r="X64" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y64" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9110,7 +9352,11 @@
       </c>
       <c r="V65" s="3" t="inlineStr"/>
       <c r="W65" s="3" t="inlineStr"/>
-      <c r="X65" s="3" t="inlineStr"/>
+      <c r="X65" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y65" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9230,7 +9476,11 @@
       </c>
       <c r="V66" s="3" t="inlineStr"/>
       <c r="W66" s="3" t="inlineStr"/>
-      <c r="X66" s="3" t="inlineStr"/>
+      <c r="X66" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9</t>
+        </is>
+      </c>
       <c r="Y66" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9350,7 +9600,11 @@
       </c>
       <c r="V67" s="3" t="inlineStr"/>
       <c r="W67" s="3" t="inlineStr"/>
-      <c r="X67" s="3" t="inlineStr"/>
+      <c r="X67" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y67" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9470,7 +9724,11 @@
       </c>
       <c r="V68" s="3" t="inlineStr"/>
       <c r="W68" s="3" t="inlineStr"/>
-      <c r="X68" s="3" t="inlineStr"/>
+      <c r="X68" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, R6</t>
+        </is>
+      </c>
       <c r="Y68" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9594,7 +9852,11 @@
       </c>
       <c r="V69" s="3" t="inlineStr"/>
       <c r="W69" s="3" t="inlineStr"/>
-      <c r="X69" s="3" t="inlineStr"/>
+      <c r="X69" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, R6</t>
+        </is>
+      </c>
       <c r="Y69" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9842,7 +10104,11 @@
       </c>
       <c r="V71" s="3" t="inlineStr"/>
       <c r="W71" s="3" t="inlineStr"/>
-      <c r="X71" s="3" t="inlineStr"/>
+      <c r="X71" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y71" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -9977,8 +10243,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA72" s="3" t="n">
-        <v>7</v>
+      <c r="AA72" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="AB72" s="3" t="inlineStr">
         <is>
@@ -10216,7 +10484,11 @@
       </c>
       <c r="V74" s="3" t="inlineStr"/>
       <c r="W74" s="3" t="inlineStr"/>
-      <c r="X74" s="3" t="inlineStr"/>
+      <c r="X74" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y74" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10336,7 +10608,11 @@
       </c>
       <c r="V75" s="3" t="inlineStr"/>
       <c r="W75" s="3" t="inlineStr"/>
-      <c r="X75" s="3" t="inlineStr"/>
+      <c r="X75" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, R9</t>
+        </is>
+      </c>
       <c r="Y75" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10456,7 +10732,11 @@
       </c>
       <c r="V76" s="3" t="inlineStr"/>
       <c r="W76" s="3" t="inlineStr"/>
-      <c r="X76" s="3" t="inlineStr"/>
+      <c r="X76" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9</t>
+        </is>
+      </c>
       <c r="Y76" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10576,7 +10856,11 @@
       </c>
       <c r="V77" s="3" t="inlineStr"/>
       <c r="W77" s="3" t="inlineStr"/>
-      <c r="X77" s="3" t="inlineStr"/>
+      <c r="X77" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y77" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10696,7 +10980,11 @@
       </c>
       <c r="V78" s="3" t="inlineStr"/>
       <c r="W78" s="3" t="inlineStr"/>
-      <c r="X78" s="3" t="inlineStr"/>
+      <c r="X78" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y78" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10816,7 +11104,11 @@
       </c>
       <c r="V79" s="3" t="inlineStr"/>
       <c r="W79" s="3" t="inlineStr"/>
-      <c r="X79" s="3" t="inlineStr"/>
+      <c r="X79" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y79" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -10936,7 +11228,11 @@
       </c>
       <c r="V80" s="3" t="inlineStr"/>
       <c r="W80" s="3" t="inlineStr"/>
-      <c r="X80" s="3" t="inlineStr"/>
+      <c r="X80" s="3" t="inlineStr">
+        <is>
+          <t>R1, R5, R7</t>
+        </is>
+      </c>
       <c r="Y80" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11056,7 +11352,11 @@
       </c>
       <c r="V81" s="3" t="inlineStr"/>
       <c r="W81" s="3" t="inlineStr"/>
-      <c r="X81" s="3" t="inlineStr"/>
+      <c r="X81" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y81" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11176,7 +11476,11 @@
       </c>
       <c r="V82" s="3" t="inlineStr"/>
       <c r="W82" s="3" t="inlineStr"/>
-      <c r="X82" s="3" t="inlineStr"/>
+      <c r="X82" s="3" t="inlineStr">
+        <is>
+          <t>R3, R7, R8</t>
+        </is>
+      </c>
       <c r="Y82" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11296,7 +11600,11 @@
       </c>
       <c r="V83" s="3" t="inlineStr"/>
       <c r="W83" s="3" t="inlineStr"/>
-      <c r="X83" s="3" t="inlineStr"/>
+      <c r="X83" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3</t>
+        </is>
+      </c>
       <c r="Y83" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11420,7 +11728,11 @@
       </c>
       <c r="V84" s="3" t="inlineStr"/>
       <c r="W84" s="3" t="inlineStr"/>
-      <c r="X84" s="3" t="inlineStr"/>
+      <c r="X84" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y84" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11544,7 +11856,11 @@
       </c>
       <c r="V85" s="3" t="inlineStr"/>
       <c r="W85" s="3" t="inlineStr"/>
-      <c r="X85" s="3" t="inlineStr"/>
+      <c r="X85" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y85" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11664,7 +11980,11 @@
       </c>
       <c r="V86" s="3" t="inlineStr"/>
       <c r="W86" s="3" t="inlineStr"/>
-      <c r="X86" s="3" t="inlineStr"/>
+      <c r="X86" s="3" t="inlineStr">
+        <is>
+          <t>R1, R5</t>
+        </is>
+      </c>
       <c r="Y86" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11784,7 +12104,11 @@
       </c>
       <c r="V87" s="3" t="inlineStr"/>
       <c r="W87" s="3" t="inlineStr"/>
-      <c r="X87" s="3" t="inlineStr"/>
+      <c r="X87" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, B1</t>
+        </is>
+      </c>
       <c r="Y87" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -11795,8 +12119,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA87" s="3" t="n">
-        <v>3</v>
+      <c r="AA87" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="AB87" s="3" t="inlineStr">
         <is>
@@ -11910,7 +12236,11 @@
       </c>
       <c r="V88" s="3" t="inlineStr"/>
       <c r="W88" s="3" t="inlineStr"/>
-      <c r="X88" s="3" t="inlineStr"/>
+      <c r="X88" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3, R6, B1</t>
+        </is>
+      </c>
       <c r="Y88" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12158,7 +12488,11 @@
       </c>
       <c r="V90" s="3" t="inlineStr"/>
       <c r="W90" s="3" t="inlineStr"/>
-      <c r="X90" s="3" t="inlineStr"/>
+      <c r="X90" s="3" t="inlineStr">
+        <is>
+          <t>R2, R9, B1</t>
+        </is>
+      </c>
       <c r="Y90" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12278,7 +12612,11 @@
       </c>
       <c r="V91" s="3" t="inlineStr"/>
       <c r="W91" s="3" t="inlineStr"/>
-      <c r="X91" s="3" t="inlineStr"/>
+      <c r="X91" s="3" t="inlineStr">
+        <is>
+          <t>R2, R6</t>
+        </is>
+      </c>
       <c r="Y91" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12406,7 +12744,11 @@
       </c>
       <c r="V92" s="3" t="inlineStr"/>
       <c r="W92" s="3" t="inlineStr"/>
-      <c r="X92" s="3" t="inlineStr"/>
+      <c r="X92" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y92" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12530,7 +12872,11 @@
       </c>
       <c r="V93" s="3" t="inlineStr"/>
       <c r="W93" s="3" t="inlineStr"/>
-      <c r="X93" s="3" t="inlineStr"/>
+      <c r="X93" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, B2</t>
+        </is>
+      </c>
       <c r="Y93" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12541,8 +12887,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA93" s="3" t="n">
-        <v>1</v>
+      <c r="AA93" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="AB93" s="3" t="inlineStr">
         <is>
@@ -12660,7 +13008,11 @@
       </c>
       <c r="V94" s="3" t="inlineStr"/>
       <c r="W94" s="3" t="inlineStr"/>
-      <c r="X94" s="3" t="inlineStr"/>
+      <c r="X94" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, B2</t>
+        </is>
+      </c>
       <c r="Y94" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12784,7 +13136,11 @@
       </c>
       <c r="V95" s="3" t="inlineStr"/>
       <c r="W95" s="3" t="inlineStr"/>
-      <c r="X95" s="3" t="inlineStr"/>
+      <c r="X95" s="3" t="inlineStr">
+        <is>
+          <t>R2, R6, B2</t>
+        </is>
+      </c>
       <c r="Y95" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12912,7 +13268,11 @@
       </c>
       <c r="V96" s="3" t="inlineStr"/>
       <c r="W96" s="3" t="inlineStr"/>
-      <c r="X96" s="3" t="inlineStr"/>
+      <c r="X96" s="3" t="inlineStr">
+        <is>
+          <t>R5, R8, R9</t>
+        </is>
+      </c>
       <c r="Y96" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -12923,8 +13283,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA96" s="3" t="n">
-        <v>2</v>
+      <c r="AA96" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="AB96" s="3" t="inlineStr">
         <is>
@@ -13042,7 +13404,11 @@
       </c>
       <c r="V97" s="3" t="inlineStr"/>
       <c r="W97" s="3" t="inlineStr"/>
-      <c r="X97" s="3" t="inlineStr"/>
+      <c r="X97" s="3" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
       <c r="Y97" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -13162,7 +13528,11 @@
       </c>
       <c r="V98" s="3" t="inlineStr"/>
       <c r="W98" s="3" t="inlineStr"/>
-      <c r="X98" s="3" t="inlineStr"/>
+      <c r="X98" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, B2</t>
+        </is>
+      </c>
       <c r="Y98" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -13286,7 +13656,11 @@
       </c>
       <c r="V99" s="3" t="inlineStr"/>
       <c r="W99" s="3" t="inlineStr"/>
-      <c r="X99" s="3" t="inlineStr"/>
+      <c r="X99" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, R3, R4, R5</t>
+        </is>
+      </c>
       <c r="Y99" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -13406,7 +13780,11 @@
       </c>
       <c r="V100" s="3" t="inlineStr"/>
       <c r="W100" s="3" t="inlineStr"/>
-      <c r="X100" s="3" t="inlineStr"/>
+      <c r="X100" s="3" t="inlineStr">
+        <is>
+          <t>R3, R10</t>
+        </is>
+      </c>
       <c r="Y100" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -13417,8 +13795,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA100" s="3" t="n">
-        <v>4</v>
+      <c r="AA100" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="AB100" s="3" t="inlineStr">
         <is>
@@ -13532,7 +13912,11 @@
       </c>
       <c r="V101" s="3" t="inlineStr"/>
       <c r="W101" s="3" t="inlineStr"/>
-      <c r="X101" s="3" t="inlineStr"/>
+      <c r="X101" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y101" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -13704,7 +14088,7 @@
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
@@ -13985,7 +14369,11 @@
       </c>
       <c r="V2" s="3" t="inlineStr"/>
       <c r="W2" s="3" t="inlineStr"/>
-      <c r="X2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>R1, R3, R7, B1</t>
+        </is>
+      </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14113,7 +14501,11 @@
       </c>
       <c r="V3" s="3" t="inlineStr"/>
       <c r="W3" s="3" t="inlineStr"/>
-      <c r="X3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2</t>
+        </is>
+      </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14241,7 +14633,11 @@
       </c>
       <c r="V4" s="3" t="inlineStr"/>
       <c r="W4" s="3" t="inlineStr"/>
-      <c r="X4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>R9, R2</t>
+        </is>
+      </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14369,7 +14765,11 @@
       </c>
       <c r="V5" s="3" t="inlineStr"/>
       <c r="W5" s="3" t="inlineStr"/>
-      <c r="X5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>R3, R7</t>
+        </is>
+      </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14497,7 +14897,11 @@
       </c>
       <c r="V6" s="3" t="inlineStr"/>
       <c r="W6" s="3" t="inlineStr"/>
-      <c r="X6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>R9, R3, R5, R8, B5, B1</t>
+        </is>
+      </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14625,7 +15029,11 @@
       </c>
       <c r="V7" s="3" t="inlineStr"/>
       <c r="W7" s="3" t="inlineStr"/>
-      <c r="X7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>R1, R4</t>
+        </is>
+      </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14753,7 +15161,11 @@
       </c>
       <c r="V8" s="3" t="inlineStr"/>
       <c r="W8" s="3" t="inlineStr"/>
-      <c r="X8" s="3" t="inlineStr"/>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>R1, B2</t>
+        </is>
+      </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -14881,7 +15293,11 @@
       </c>
       <c r="V9" s="3" t="inlineStr"/>
       <c r="W9" s="3" t="inlineStr"/>
-      <c r="X9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>R4, R7, R9</t>
+        </is>
+      </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -15009,7 +15425,11 @@
       </c>
       <c r="V10" s="3" t="inlineStr"/>
       <c r="W10" s="3" t="inlineStr"/>
-      <c r="X10" s="3" t="inlineStr"/>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
+          <t>R9, R6</t>
+        </is>
+      </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -15137,7 +15557,11 @@
       </c>
       <c r="V11" s="3" t="inlineStr"/>
       <c r="W11" s="3" t="inlineStr"/>
-      <c r="X11" s="3" t="inlineStr"/>
+      <c r="X11" s="3" t="inlineStr">
+        <is>
+          <t>R1, R9, R2</t>
+        </is>
+      </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -15265,7 +15689,11 @@
       </c>
       <c r="V12" s="3" t="inlineStr"/>
       <c r="W12" s="3" t="inlineStr"/>
-      <c r="X12" s="3" t="inlineStr"/>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>R10, R9</t>
+        </is>
+      </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -15393,7 +15821,11 @@
       </c>
       <c r="V13" s="3" t="inlineStr"/>
       <c r="W13" s="3" t="inlineStr"/>
-      <c r="X13" s="3" t="inlineStr"/>
+      <c r="X13" s="3" t="inlineStr">
+        <is>
+          <t>R1, R2, B1</t>
+        </is>
+      </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -15517,7 +15949,11 @@
       </c>
       <c r="V14" s="3" t="inlineStr"/>
       <c r="W14" s="3" t="inlineStr"/>
-      <c r="X14" s="3" t="inlineStr"/>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, B2</t>
+        </is>
+      </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -15528,8 +15964,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA14" s="3" t="n">
-        <v>1</v>
+      <c r="AA14" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="AB14" s="3" t="inlineStr">
         <is>
@@ -15651,7 +16089,11 @@
       </c>
       <c r="V15" s="3" t="inlineStr"/>
       <c r="W15" s="3" t="inlineStr"/>
-      <c r="X15" s="3" t="inlineStr"/>
+      <c r="X15" s="3" t="inlineStr">
+        <is>
+          <t>R5, R8, R9</t>
+        </is>
+      </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -15662,8 +16104,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA15" s="3" t="n">
-        <v>2</v>
+      <c r="AA15" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="AB15" s="3" t="inlineStr">
         <is>
@@ -15781,7 +16225,11 @@
       </c>
       <c r="V16" s="3" t="inlineStr"/>
       <c r="W16" s="3" t="inlineStr"/>
-      <c r="X16" s="3" t="inlineStr"/>
+      <c r="X16" s="3" t="inlineStr">
+        <is>
+          <t>R1, R6, B1</t>
+        </is>
+      </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -15792,8 +16240,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA16" s="3" t="n">
-        <v>3</v>
+      <c r="AA16" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="AB16" s="3" t="inlineStr">
         <is>
@@ -15907,7 +16357,11 @@
       </c>
       <c r="V17" s="3" t="inlineStr"/>
       <c r="W17" s="3" t="inlineStr"/>
-      <c r="X17" s="3" t="inlineStr"/>
+      <c r="X17" s="3" t="inlineStr">
+        <is>
+          <t>R3, R10</t>
+        </is>
+      </c>
       <c r="Y17" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -15918,8 +16372,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA17" s="3" t="n">
-        <v>4</v>
+      <c r="AA17" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="AB17" s="3" t="inlineStr">
         <is>
@@ -16037,7 +16493,11 @@
       </c>
       <c r="V18" s="3" t="inlineStr"/>
       <c r="W18" s="3" t="inlineStr"/>
-      <c r="X18" s="3" t="inlineStr"/>
+      <c r="X18" s="3" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -16048,8 +16508,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA18" s="3" t="n">
-        <v>5</v>
+      <c r="AA18" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="AB18" s="3" t="inlineStr">
         <is>
@@ -16171,7 +16633,11 @@
       </c>
       <c r="V19" s="3" t="inlineStr"/>
       <c r="W19" s="3" t="inlineStr"/>
-      <c r="X19" s="3" t="inlineStr"/>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
       <c r="Y19" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -16182,8 +16648,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA19" s="3" t="n">
-        <v>6</v>
+      <c r="AA19" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="AB19" s="3" t="inlineStr">
         <is>
@@ -16316,8 +16784,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA20" s="3" t="n">
-        <v>7</v>
+      <c r="AA20" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="AB20" s="3" t="inlineStr">
         <is>
@@ -16431,7 +16901,11 @@
       </c>
       <c r="V21" s="3" t="inlineStr"/>
       <c r="W21" s="3" t="inlineStr"/>
-      <c r="X21" s="3" t="inlineStr"/>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
       <c r="Y21" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -16442,8 +16916,10 @@
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="AA21" s="3" t="n">
-        <v>8</v>
+      <c r="AA21" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="AB21" s="3" t="inlineStr">
         <is>
@@ -16814,7 +17290,11 @@
       </c>
       <c r="V2" s="3" t="inlineStr"/>
       <c r="W2" s="3" t="inlineStr"/>
-      <c r="X2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -16950,7 +17430,11 @@
       </c>
       <c r="V3" s="3" t="inlineStr"/>
       <c r="W3" s="3" t="inlineStr"/>
-      <c r="X3" s="3" t="inlineStr"/>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17086,7 +17570,11 @@
       </c>
       <c r="V4" s="3" t="inlineStr"/>
       <c r="W4" s="3" t="inlineStr"/>
-      <c r="X4" s="3" t="inlineStr"/>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17222,7 +17710,11 @@
       </c>
       <c r="V5" s="3" t="inlineStr"/>
       <c r="W5" s="3" t="inlineStr"/>
-      <c r="X5" s="3" t="inlineStr"/>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17354,7 +17846,11 @@
       </c>
       <c r="V6" s="3" t="inlineStr"/>
       <c r="W6" s="3" t="inlineStr"/>
-      <c r="X6" s="3" t="inlineStr"/>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17478,7 +17974,11 @@
       </c>
       <c r="V7" s="3" t="inlineStr"/>
       <c r="W7" s="3" t="inlineStr"/>
-      <c r="X7" s="3" t="inlineStr"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17602,7 +18102,11 @@
       </c>
       <c r="V8" s="3" t="inlineStr"/>
       <c r="W8" s="3" t="inlineStr"/>
-      <c r="X8" s="3" t="inlineStr"/>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
           <t>no</t>
@@ -17730,7 +18234,11 @@
       </c>
       <c r="V9" s="3" t="inlineStr"/>
       <c r="W9" s="3" t="inlineStr"/>
-      <c r="X9" s="3" t="inlineStr"/>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
           <t>no</t>

</xml_diff>

<commit_message>
E1: combined 20-case summary and redrafted E1 manuscript section
- E1_SUMMARY.md (make_e1_summary.py, reads recorded results only): depth 20 cases
  (Stage A 12 + depth v2 8), 53/53 histories exact, corpus 92/6/2/0, R/B counts
- Evaluation PerCom_version.md: E1 section rewritten as a draft pending author review
  (source-diverse corpus, fixed screening sentence, scoped verdicts, no extractor,
  finite-state, general-accumulator or concurrency overclaims)
- Limitations HANDOFF: item 3 separates depth and corpus counts; extractor item removed
- workbook codebook: class columns marked preliminary, not reconciled with rb_adjudicated

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPrygyUUKfHFM8zKEvmbin
</commit_message>
<xml_diff>
--- a/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
+++ b/PerCom/6_Evaluation/E1_adequacy/breadth/E1_CORPUS_WORKBOOK.xlsx
@@ -23863,7 +23863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24005,34 +24005,46 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>text_form</t>
+          <t>trigger_class / temporal_class / control_class / memory_class / action_cardinality / lifetime</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Whether text is verbatim, source-extracted, or researcher-normalized.</t>
+          <t>Preliminary machine-assisted descriptors. Only the corrections the author stated on 2026-09-13 were applied; they are not reconciled with rb_adjudicated and are not used in any statistic.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>completed_seed</t>
+          <t>text_form</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>One of the existing 12 depth cases.</t>
+          <t>Whether text is verbatim, source-extracted, or researcher-normalized.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>completed_seed</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>One of the existing 12 depth cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>proposed_depth_addition</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>One of the eight new depth cases (final selection; value name kept for file compatibility). Results: depth/RESULTS.md.</t>
         </is>

</xml_diff>